<commit_message>
Add trails, parks (federal ABA), polling places and festival areas
Trails, wetland boardwalks, park paths, beaches, picnic, camping and
overlooks are checked against ABA Chapter 10: required when the visit
records federal funds, best practice when not, manual when unknown.
Polling place visits follow the DOJ ADA Checklist for Polling Places,
with voting station and temporary fix checks. Festival or event areas
cover tents and booths, event paths and cable covers, and portable
toilets.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AdurZhc4WrEcjZAJU4UBbC
</commit_message>
<xml_diff>
--- a/Rules review - Michigan citations to verify.xlsx
+++ b/Rules review - Michigan citations to verify.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L180"/>
+  <dimension ref="A1:L257"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -484,12 +484,12 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>ADA 2010 citation</t>
+          <t>Federal citation (ADA 2010, ABA, HAVA)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>ADA 2010 limit</t>
+          <t>Federal limit</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -509,7 +509,7 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Michigan citation correct? (Y/N)</t>
+          <t>Citations correct? (Y/N)</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
@@ -8142,13 +8142,3007 @@
       <c r="G180" s="2" t="n"/>
       <c r="H180" s="2" t="inlineStr">
         <is>
-          <t>The 2010 ADA Standards have no picnic-table or park-bench rules; dining-surface rules (5% accessible) are applied here by practice. Federal outdoor areas follow ABA Chapter 10 instead.</t>
+          <t>The 2010 ADA Standards have no picnic-table or park-bench rules; dining-surface rules (5% accessible) are applied here by practice. For park picnic tables under the federal ABA rules, record "Picnic table (park or picnic area)".</t>
         </is>
       </c>
       <c r="I180" s="2" t="n"/>
       <c r="J180" s="2" t="n"/>
       <c r="K180" s="2" t="n"/>
       <c r="L180" s="2" t="n"/>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="inlineStr">
+        <is>
+          <t>Trail, nature path or wetland boardwalk</t>
+        </is>
+      </c>
+      <c r="B181" s="2" t="inlineStr">
+        <is>
+          <t>Firm and stable surface</t>
+        </is>
+      </c>
+      <c r="C181" s="2" t="inlineStr">
+        <is>
+          <t>yes/no</t>
+        </is>
+      </c>
+      <c r="D181" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1017.3</t>
+        </is>
+      </c>
+      <c r="E181" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F181" s="2" t="n"/>
+      <c r="G181" s="2" t="n"/>
+      <c r="H181" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I181" s="2" t="n"/>
+      <c r="J181" s="2" t="n"/>
+      <c r="K181" s="2" t="n"/>
+      <c r="L181" s="2" t="n"/>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
+        <is>
+          <t>Trail, nature path or wetland boardwalk</t>
+        </is>
+      </c>
+      <c r="B182" s="2" t="inlineStr">
+        <is>
+          <t>Clear tread width (36 in min)</t>
+        </is>
+      </c>
+      <c r="C182" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D182" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1017.4</t>
+        </is>
+      </c>
+      <c r="E182" s="2" t="inlineStr">
+        <is>
+          <t>min 36</t>
+        </is>
+      </c>
+      <c r="F182" s="2" t="n"/>
+      <c r="G182" s="2" t="n"/>
+      <c r="H182" s="2" t="inlineStr">
+        <is>
+          <t>May narrow to 32 in where there is a physical constraint. Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I182" s="2" t="n"/>
+      <c r="J182" s="2" t="n"/>
+      <c r="K182" s="2" t="n"/>
+      <c r="L182" s="2" t="n"/>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="inlineStr">
+        <is>
+          <t>Trail, nature path or wetland boardwalk</t>
+        </is>
+      </c>
+      <c r="B183" s="2" t="inlineStr">
+        <is>
+          <t>Passing spaces</t>
+        </is>
+      </c>
+      <c r="C183" s="2" t="inlineStr">
+        <is>
+          <t>yes/no</t>
+        </is>
+      </c>
+      <c r="D183" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1017.5</t>
+        </is>
+      </c>
+      <c r="E183" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F183" s="2" t="n"/>
+      <c r="G183" s="2" t="n"/>
+      <c r="H183" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I183" s="2" t="n"/>
+      <c r="J183" s="2" t="n"/>
+      <c r="K183" s="2" t="n"/>
+      <c r="L183" s="2" t="n"/>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
+        <is>
+          <t>Trail, nature path or wetland boardwalk</t>
+        </is>
+      </c>
+      <c r="B184" s="2" t="inlineStr">
+        <is>
+          <t>Tread obstacles (2 in max)</t>
+        </is>
+      </c>
+      <c r="C184" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D184" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1017.6</t>
+        </is>
+      </c>
+      <c r="E184" s="2" t="inlineStr">
+        <is>
+          <t>max 2</t>
+        </is>
+      </c>
+      <c r="F184" s="2" t="n"/>
+      <c r="G184" s="2" t="n"/>
+      <c r="H184" s="2" t="inlineStr">
+        <is>
+          <t>Up to 3 in is allowed where running and cross slopes are 1:20 or less. Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I184" s="2" t="n"/>
+      <c r="J184" s="2" t="n"/>
+      <c r="K184" s="2" t="n"/>
+      <c r="L184" s="2" t="n"/>
+    </row>
+    <row r="185">
+      <c r="A185" s="2" t="inlineStr">
+        <is>
+          <t>Trail, nature path or wetland boardwalk</t>
+        </is>
+      </c>
+      <c r="B185" s="2" t="inlineStr">
+        <is>
+          <t>Openings (1/2 in max)</t>
+        </is>
+      </c>
+      <c r="C185" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D185" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1017.7</t>
+        </is>
+      </c>
+      <c r="E185" s="2" t="inlineStr">
+        <is>
+          <t>max 0.5</t>
+        </is>
+      </c>
+      <c r="F185" s="2" t="n"/>
+      <c r="G185" s="2" t="n"/>
+      <c r="H185" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I185" s="2" t="n"/>
+      <c r="J185" s="2" t="n"/>
+      <c r="K185" s="2" t="n"/>
+      <c r="L185" s="2" t="n"/>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
+        <is>
+          <t>Trail, nature path or wetland boardwalk</t>
+        </is>
+      </c>
+      <c r="B186" s="2" t="inlineStr">
+        <is>
+          <t>Running slope and segment length</t>
+        </is>
+      </c>
+      <c r="C186" s="2" t="inlineStr">
+        <is>
+          <t>abaSlope</t>
+        </is>
+      </c>
+      <c r="D186" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1017.8.1</t>
+        </is>
+      </c>
+      <c r="E186" s="2" t="n"/>
+      <c r="F186" s="2" t="n"/>
+      <c r="G186" s="2" t="n"/>
+      <c r="H186" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I186" s="2" t="n"/>
+      <c r="J186" s="2" t="n"/>
+      <c r="K186" s="2" t="n"/>
+      <c r="L186" s="2" t="n"/>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="inlineStr">
+        <is>
+          <t>Trail, nature path or wetland boardwalk</t>
+        </is>
+      </c>
+      <c r="B187" s="2" t="inlineStr">
+        <is>
+          <t>No more than 30% of the trail steeper than 1:12</t>
+        </is>
+      </c>
+      <c r="C187" s="2" t="inlineStr">
+        <is>
+          <t>yes/no</t>
+        </is>
+      </c>
+      <c r="D187" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1017.8.1</t>
+        </is>
+      </c>
+      <c r="E187" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F187" s="2" t="n"/>
+      <c r="G187" s="2" t="n"/>
+      <c r="H187" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I187" s="2" t="n"/>
+      <c r="J187" s="2" t="n"/>
+      <c r="K187" s="2" t="n"/>
+      <c r="L187" s="2" t="n"/>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="inlineStr">
+        <is>
+          <t>Trail, nature path or wetland boardwalk</t>
+        </is>
+      </c>
+      <c r="B188" s="2" t="inlineStr">
+        <is>
+          <t>Cross slope (1:20 max)</t>
+        </is>
+      </c>
+      <c r="C188" s="2" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D188" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1017.8.2</t>
+        </is>
+      </c>
+      <c r="E188" s="2" t="inlineStr">
+        <is>
+          <t>max 5</t>
+        </is>
+      </c>
+      <c r="F188" s="2" t="n"/>
+      <c r="G188" s="2" t="n"/>
+      <c r="H188" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I188" s="2" t="n"/>
+      <c r="J188" s="2" t="n"/>
+      <c r="K188" s="2" t="n"/>
+      <c r="L188" s="2" t="n"/>
+    </row>
+    <row r="189">
+      <c r="A189" s="2" t="inlineStr">
+        <is>
+          <t>Trail, nature path or wetland boardwalk</t>
+        </is>
+      </c>
+      <c r="B189" s="2" t="inlineStr">
+        <is>
+          <t>Resting intervals</t>
+        </is>
+      </c>
+      <c r="C189" s="2" t="inlineStr">
+        <is>
+          <t>yes/no</t>
+        </is>
+      </c>
+      <c r="D189" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1017.9</t>
+        </is>
+      </c>
+      <c r="E189" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F189" s="2" t="n"/>
+      <c r="G189" s="2" t="n"/>
+      <c r="H189" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I189" s="2" t="n"/>
+      <c r="J189" s="2" t="n"/>
+      <c r="K189" s="2" t="n"/>
+      <c r="L189" s="2" t="n"/>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="inlineStr">
+        <is>
+          <t>Trail, nature path or wetland boardwalk</t>
+        </is>
+      </c>
+      <c r="B190" s="2" t="inlineStr">
+        <is>
+          <t>Headroom (80 in min)</t>
+        </is>
+      </c>
+      <c r="C190" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D190" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1017.10</t>
+        </is>
+      </c>
+      <c r="E190" s="2" t="inlineStr">
+        <is>
+          <t>min 80</t>
+        </is>
+      </c>
+      <c r="F190" s="2" t="n"/>
+      <c r="G190" s="2" t="n"/>
+      <c r="H190" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I190" s="2" t="n"/>
+      <c r="J190" s="2" t="n"/>
+      <c r="K190" s="2" t="n"/>
+      <c r="L190" s="2" t="n"/>
+    </row>
+    <row r="191">
+      <c r="A191" s="2" t="inlineStr">
+        <is>
+          <t>Trail, nature path or wetland boardwalk</t>
+        </is>
+      </c>
+      <c r="B191" s="2" t="inlineStr">
+        <is>
+          <t>Trailhead signs</t>
+        </is>
+      </c>
+      <c r="C191" s="2" t="inlineStr">
+        <is>
+          <t>yes/no</t>
+        </is>
+      </c>
+      <c r="D191" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1017.11</t>
+        </is>
+      </c>
+      <c r="E191" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F191" s="2" t="n"/>
+      <c r="G191" s="2" t="n"/>
+      <c r="H191" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I191" s="2" t="n"/>
+      <c r="J191" s="2" t="n"/>
+      <c r="K191" s="2" t="n"/>
+      <c r="L191" s="2" t="n"/>
+    </row>
+    <row r="192">
+      <c r="A192" s="2" t="inlineStr">
+        <is>
+          <t>Outdoor recreation access route (park path)</t>
+        </is>
+      </c>
+      <c r="B192" s="2" t="inlineStr">
+        <is>
+          <t>Firm and stable surface</t>
+        </is>
+      </c>
+      <c r="C192" s="2" t="inlineStr">
+        <is>
+          <t>yes/no</t>
+        </is>
+      </c>
+      <c r="D192" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1016.2</t>
+        </is>
+      </c>
+      <c r="E192" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F192" s="2" t="n"/>
+      <c r="G192" s="2" t="n"/>
+      <c r="H192" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I192" s="2" t="n"/>
+      <c r="J192" s="2" t="n"/>
+      <c r="K192" s="2" t="n"/>
+      <c r="L192" s="2" t="n"/>
+    </row>
+    <row r="193">
+      <c r="A193" s="2" t="inlineStr">
+        <is>
+          <t>Outdoor recreation access route (park path)</t>
+        </is>
+      </c>
+      <c r="B193" s="2" t="inlineStr">
+        <is>
+          <t>Clear tread width (36 in min)</t>
+        </is>
+      </c>
+      <c r="C193" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D193" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1016.3</t>
+        </is>
+      </c>
+      <c r="E193" s="2" t="inlineStr">
+        <is>
+          <t>min 36</t>
+        </is>
+      </c>
+      <c r="F193" s="2" t="n"/>
+      <c r="G193" s="2" t="n"/>
+      <c r="H193" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I193" s="2" t="n"/>
+      <c r="J193" s="2" t="n"/>
+      <c r="K193" s="2" t="n"/>
+      <c r="L193" s="2" t="n"/>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="inlineStr">
+        <is>
+          <t>Outdoor recreation access route (park path)</t>
+        </is>
+      </c>
+      <c r="B194" s="2" t="inlineStr">
+        <is>
+          <t>Passing spaces</t>
+        </is>
+      </c>
+      <c r="C194" s="2" t="inlineStr">
+        <is>
+          <t>yes/no</t>
+        </is>
+      </c>
+      <c r="D194" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1016.4</t>
+        </is>
+      </c>
+      <c r="E194" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F194" s="2" t="n"/>
+      <c r="G194" s="2" t="n"/>
+      <c r="H194" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I194" s="2" t="n"/>
+      <c r="J194" s="2" t="n"/>
+      <c r="K194" s="2" t="n"/>
+      <c r="L194" s="2" t="n"/>
+    </row>
+    <row r="195">
+      <c r="A195" s="2" t="inlineStr">
+        <is>
+          <t>Outdoor recreation access route (park path)</t>
+        </is>
+      </c>
+      <c r="B195" s="2" t="inlineStr">
+        <is>
+          <t>Tread obstacles (1/2 in max)</t>
+        </is>
+      </c>
+      <c r="C195" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D195" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1016.5</t>
+        </is>
+      </c>
+      <c r="E195" s="2" t="inlineStr">
+        <is>
+          <t>max 0.5</t>
+        </is>
+      </c>
+      <c r="F195" s="2" t="n"/>
+      <c r="G195" s="2" t="n"/>
+      <c r="H195" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I195" s="2" t="n"/>
+      <c r="J195" s="2" t="n"/>
+      <c r="K195" s="2" t="n"/>
+      <c r="L195" s="2" t="n"/>
+    </row>
+    <row r="196">
+      <c r="A196" s="2" t="inlineStr">
+        <is>
+          <t>Outdoor recreation access route (park path)</t>
+        </is>
+      </c>
+      <c r="B196" s="2" t="inlineStr">
+        <is>
+          <t>Openings (1/2 in max)</t>
+        </is>
+      </c>
+      <c r="C196" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D196" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1016.6</t>
+        </is>
+      </c>
+      <c r="E196" s="2" t="inlineStr">
+        <is>
+          <t>max 0.5</t>
+        </is>
+      </c>
+      <c r="F196" s="2" t="n"/>
+      <c r="G196" s="2" t="n"/>
+      <c r="H196" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I196" s="2" t="n"/>
+      <c r="J196" s="2" t="n"/>
+      <c r="K196" s="2" t="n"/>
+      <c r="L196" s="2" t="n"/>
+    </row>
+    <row r="197">
+      <c r="A197" s="2" t="inlineStr">
+        <is>
+          <t>Outdoor recreation access route (park path)</t>
+        </is>
+      </c>
+      <c r="B197" s="2" t="inlineStr">
+        <is>
+          <t>Running slope and segment length</t>
+        </is>
+      </c>
+      <c r="C197" s="2" t="inlineStr">
+        <is>
+          <t>abaSlope</t>
+        </is>
+      </c>
+      <c r="D197" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1016.7.1</t>
+        </is>
+      </c>
+      <c r="E197" s="2" t="n"/>
+      <c r="F197" s="2" t="n"/>
+      <c r="G197" s="2" t="n"/>
+      <c r="H197" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I197" s="2" t="n"/>
+      <c r="J197" s="2" t="n"/>
+      <c r="K197" s="2" t="n"/>
+      <c r="L197" s="2" t="n"/>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="inlineStr">
+        <is>
+          <t>Outdoor recreation access route (park path)</t>
+        </is>
+      </c>
+      <c r="B198" s="2" t="inlineStr">
+        <is>
+          <t>Cross slope (1:33 max)</t>
+        </is>
+      </c>
+      <c r="C198" s="2" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D198" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1016.7.2</t>
+        </is>
+      </c>
+      <c r="E198" s="2" t="inlineStr">
+        <is>
+          <t>max 3.03</t>
+        </is>
+      </c>
+      <c r="F198" s="2" t="n"/>
+      <c r="G198" s="2" t="n"/>
+      <c r="H198" s="2" t="inlineStr">
+        <is>
+          <t>Up to 1:20 is allowed on surfaces other than asphalt, concrete and boards where needed for drainage. Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I198" s="2" t="n"/>
+      <c r="J198" s="2" t="n"/>
+      <c r="K198" s="2" t="n"/>
+      <c r="L198" s="2" t="n"/>
+    </row>
+    <row r="199">
+      <c r="A199" s="2" t="inlineStr">
+        <is>
+          <t>Outdoor recreation access route (park path)</t>
+        </is>
+      </c>
+      <c r="B199" s="2" t="inlineStr">
+        <is>
+          <t>Resting intervals</t>
+        </is>
+      </c>
+      <c r="C199" s="2" t="inlineStr">
+        <is>
+          <t>yes/no</t>
+        </is>
+      </c>
+      <c r="D199" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1016.8</t>
+        </is>
+      </c>
+      <c r="E199" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F199" s="2" t="n"/>
+      <c r="G199" s="2" t="n"/>
+      <c r="H199" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I199" s="2" t="n"/>
+      <c r="J199" s="2" t="n"/>
+      <c r="K199" s="2" t="n"/>
+      <c r="L199" s="2" t="n"/>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="inlineStr">
+        <is>
+          <t>Outdoor recreation access route (park path)</t>
+        </is>
+      </c>
+      <c r="B200" s="2" t="inlineStr">
+        <is>
+          <t>Headroom (80 in min)</t>
+        </is>
+      </c>
+      <c r="C200" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D200" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1016.9</t>
+        </is>
+      </c>
+      <c r="E200" s="2" t="inlineStr">
+        <is>
+          <t>min 80</t>
+        </is>
+      </c>
+      <c r="F200" s="2" t="n"/>
+      <c r="G200" s="2" t="n"/>
+      <c r="H200" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I200" s="2" t="n"/>
+      <c r="J200" s="2" t="n"/>
+      <c r="K200" s="2" t="n"/>
+      <c r="L200" s="2" t="n"/>
+    </row>
+    <row r="201">
+      <c r="A201" s="2" t="inlineStr">
+        <is>
+          <t>Beach access route</t>
+        </is>
+      </c>
+      <c r="B201" s="2" t="inlineStr">
+        <is>
+          <t>Firm and stable surface</t>
+        </is>
+      </c>
+      <c r="C201" s="2" t="inlineStr">
+        <is>
+          <t>yes/no</t>
+        </is>
+      </c>
+      <c r="D201" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1018.3</t>
+        </is>
+      </c>
+      <c r="E201" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F201" s="2" t="n"/>
+      <c r="G201" s="2" t="n"/>
+      <c r="H201" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I201" s="2" t="n"/>
+      <c r="J201" s="2" t="n"/>
+      <c r="K201" s="2" t="n"/>
+      <c r="L201" s="2" t="n"/>
+    </row>
+    <row r="202">
+      <c r="A202" s="2" t="inlineStr">
+        <is>
+          <t>Beach access route</t>
+        </is>
+      </c>
+      <c r="B202" s="2" t="inlineStr">
+        <is>
+          <t>Clear width (60 in min)</t>
+        </is>
+      </c>
+      <c r="C202" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D202" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1018.4</t>
+        </is>
+      </c>
+      <c r="E202" s="2" t="inlineStr">
+        <is>
+          <t>min 60</t>
+        </is>
+      </c>
+      <c r="F202" s="2" t="n"/>
+      <c r="G202" s="2" t="n"/>
+      <c r="H202" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I202" s="2" t="n"/>
+      <c r="J202" s="2" t="n"/>
+      <c r="K202" s="2" t="n"/>
+      <c r="L202" s="2" t="n"/>
+    </row>
+    <row r="203">
+      <c r="A203" s="2" t="inlineStr">
+        <is>
+          <t>Beach access route</t>
+        </is>
+      </c>
+      <c r="B203" s="2" t="inlineStr">
+        <is>
+          <t>Running slope and segment length</t>
+        </is>
+      </c>
+      <c r="C203" s="2" t="inlineStr">
+        <is>
+          <t>abaSlope</t>
+        </is>
+      </c>
+      <c r="D203" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1018.7.1</t>
+        </is>
+      </c>
+      <c r="E203" s="2" t="n"/>
+      <c r="F203" s="2" t="n"/>
+      <c r="G203" s="2" t="n"/>
+      <c r="H203" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I203" s="2" t="n"/>
+      <c r="J203" s="2" t="n"/>
+      <c r="K203" s="2" t="n"/>
+      <c r="L203" s="2" t="n"/>
+    </row>
+    <row r="204">
+      <c r="A204" s="2" t="inlineStr">
+        <is>
+          <t>Beach access route</t>
+        </is>
+      </c>
+      <c r="B204" s="2" t="inlineStr">
+        <is>
+          <t>Cross slope (1:50 max)</t>
+        </is>
+      </c>
+      <c r="C204" s="2" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D204" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1018.7.2</t>
+        </is>
+      </c>
+      <c r="E204" s="2" t="inlineStr">
+        <is>
+          <t>max 2</t>
+        </is>
+      </c>
+      <c r="F204" s="2" t="n"/>
+      <c r="G204" s="2" t="n"/>
+      <c r="H204" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I204" s="2" t="n"/>
+      <c r="J204" s="2" t="n"/>
+      <c r="K204" s="2" t="n"/>
+      <c r="L204" s="2" t="n"/>
+    </row>
+    <row r="205">
+      <c r="A205" s="2" t="inlineStr">
+        <is>
+          <t>Beach access route</t>
+        </is>
+      </c>
+      <c r="B205" s="2" t="inlineStr">
+        <is>
+          <t>Obstacles (1/2 in max)</t>
+        </is>
+      </c>
+      <c r="C205" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D205" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1018.5</t>
+        </is>
+      </c>
+      <c r="E205" s="2" t="inlineStr">
+        <is>
+          <t>max 0.5</t>
+        </is>
+      </c>
+      <c r="F205" s="2" t="n"/>
+      <c r="G205" s="2" t="n"/>
+      <c r="H205" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I205" s="2" t="n"/>
+      <c r="J205" s="2" t="n"/>
+      <c r="K205" s="2" t="n"/>
+      <c r="L205" s="2" t="n"/>
+    </row>
+    <row r="206">
+      <c r="A206" s="2" t="inlineStr">
+        <is>
+          <t>Beach access route</t>
+        </is>
+      </c>
+      <c r="B206" s="2" t="inlineStr">
+        <is>
+          <t>Reaches the water</t>
+        </is>
+      </c>
+      <c r="C206" s="2" t="inlineStr">
+        <is>
+          <t>yes/no</t>
+        </is>
+      </c>
+      <c r="D206" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1018.2</t>
+        </is>
+      </c>
+      <c r="E206" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F206" s="2" t="n"/>
+      <c r="G206" s="2" t="n"/>
+      <c r="H206" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I206" s="2" t="n"/>
+      <c r="J206" s="2" t="n"/>
+      <c r="K206" s="2" t="n"/>
+      <c r="L206" s="2" t="n"/>
+    </row>
+    <row r="207">
+      <c r="A207" s="2" t="inlineStr">
+        <is>
+          <t>Picnic table (park or picnic area)</t>
+        </is>
+      </c>
+      <c r="B207" s="2" t="inlineStr">
+        <is>
+          <t>At least 20% of tables accessible</t>
+        </is>
+      </c>
+      <c r="C207" s="2" t="inlineStr">
+        <is>
+          <t>ratio</t>
+        </is>
+      </c>
+      <c r="D207" s="2" t="inlineStr">
+        <is>
+          <t>ABA §F245.2.1</t>
+        </is>
+      </c>
+      <c r="E207" s="2" t="n"/>
+      <c r="F207" s="2" t="n"/>
+      <c r="G207" s="2" t="n"/>
+      <c r="H207" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I207" s="2" t="n"/>
+      <c r="J207" s="2" t="n"/>
+      <c r="K207" s="2" t="n"/>
+      <c r="L207" s="2" t="n"/>
+    </row>
+    <row r="208">
+      <c r="A208" s="2" t="inlineStr">
+        <is>
+          <t>Picnic table (park or picnic area)</t>
+        </is>
+      </c>
+      <c r="B208" s="2" t="inlineStr">
+        <is>
+          <t>Table top height (28 to 34 in)</t>
+        </is>
+      </c>
+      <c r="C208" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D208" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1011.3.1</t>
+        </is>
+      </c>
+      <c r="E208" s="2" t="inlineStr">
+        <is>
+          <t>min 28, max 34</t>
+        </is>
+      </c>
+      <c r="F208" s="2" t="n"/>
+      <c r="G208" s="2" t="n"/>
+      <c r="H208" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I208" s="2" t="n"/>
+      <c r="J208" s="2" t="n"/>
+      <c r="K208" s="2" t="n"/>
+      <c r="L208" s="2" t="n"/>
+    </row>
+    <row r="209">
+      <c r="A209" s="2" t="inlineStr">
+        <is>
+          <t>Picnic table (park or picnic area)</t>
+        </is>
+      </c>
+      <c r="B209" s="2" t="inlineStr">
+        <is>
+          <t>Knee clearance height (27 in min)</t>
+        </is>
+      </c>
+      <c r="C209" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D209" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1011.3.2</t>
+        </is>
+      </c>
+      <c r="E209" s="2" t="inlineStr">
+        <is>
+          <t>min 27</t>
+        </is>
+      </c>
+      <c r="F209" s="2" t="n"/>
+      <c r="G209" s="2" t="n"/>
+      <c r="H209" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I209" s="2" t="n"/>
+      <c r="J209" s="2" t="n"/>
+      <c r="K209" s="2" t="n"/>
+      <c r="L209" s="2" t="n"/>
+    </row>
+    <row r="210">
+      <c r="A210" s="2" t="inlineStr">
+        <is>
+          <t>Picnic table (park or picnic area)</t>
+        </is>
+      </c>
+      <c r="B210" s="2" t="inlineStr">
+        <is>
+          <t>Knee clearance depth (19 in min)</t>
+        </is>
+      </c>
+      <c r="C210" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D210" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1011.3.2</t>
+        </is>
+      </c>
+      <c r="E210" s="2" t="inlineStr">
+        <is>
+          <t>min 19</t>
+        </is>
+      </c>
+      <c r="F210" s="2" t="n"/>
+      <c r="G210" s="2" t="n"/>
+      <c r="H210" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I210" s="2" t="n"/>
+      <c r="J210" s="2" t="n"/>
+      <c r="K210" s="2" t="n"/>
+      <c r="L210" s="2" t="n"/>
+    </row>
+    <row r="211">
+      <c r="A211" s="2" t="inlineStr">
+        <is>
+          <t>Picnic table (park or picnic area)</t>
+        </is>
+      </c>
+      <c r="B211" s="2" t="inlineStr">
+        <is>
+          <t>Clear ground space around usable sides (36 in min)</t>
+        </is>
+      </c>
+      <c r="C211" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D211" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1011.3.3</t>
+        </is>
+      </c>
+      <c r="E211" s="2" t="inlineStr">
+        <is>
+          <t>min 36</t>
+        </is>
+      </c>
+      <c r="F211" s="2" t="n"/>
+      <c r="G211" s="2" t="n"/>
+      <c r="H211" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I211" s="2" t="n"/>
+      <c r="J211" s="2" t="n"/>
+      <c r="K211" s="2" t="n"/>
+      <c r="L211" s="2" t="n"/>
+    </row>
+    <row r="212">
+      <c r="A212" s="2" t="inlineStr">
+        <is>
+          <t>Picnic table (park or picnic area)</t>
+        </is>
+      </c>
+      <c r="B212" s="2" t="inlineStr">
+        <is>
+          <t>Ground surface</t>
+        </is>
+      </c>
+      <c r="C212" s="2" t="inlineStr">
+        <is>
+          <t>yes/no</t>
+        </is>
+      </c>
+      <c r="D212" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1011.2</t>
+        </is>
+      </c>
+      <c r="E212" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F212" s="2" t="n"/>
+      <c r="G212" s="2" t="n"/>
+      <c r="H212" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I212" s="2" t="n"/>
+      <c r="J212" s="2" t="n"/>
+      <c r="K212" s="2" t="n"/>
+      <c r="L212" s="2" t="n"/>
+    </row>
+    <row r="213">
+      <c r="A213" s="2" t="inlineStr">
+        <is>
+          <t>Fire ring, grill or cooking surface</t>
+        </is>
+      </c>
+      <c r="B213" s="2" t="inlineStr">
+        <is>
+          <t>Cooking surface height (15 to 34 in)</t>
+        </is>
+      </c>
+      <c r="C213" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D213" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1011.5 and 1011.6</t>
+        </is>
+      </c>
+      <c r="E213" s="2" t="inlineStr">
+        <is>
+          <t>min 15, max 34</t>
+        </is>
+      </c>
+      <c r="F213" s="2" t="n"/>
+      <c r="G213" s="2" t="n"/>
+      <c r="H213" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I213" s="2" t="n"/>
+      <c r="J213" s="2" t="n"/>
+      <c r="K213" s="2" t="n"/>
+      <c r="L213" s="2" t="n"/>
+    </row>
+    <row r="214">
+      <c r="A214" s="2" t="inlineStr">
+        <is>
+          <t>Fire ring, grill or cooking surface</t>
+        </is>
+      </c>
+      <c r="B214" s="2" t="inlineStr">
+        <is>
+          <t>Clear ground space</t>
+        </is>
+      </c>
+      <c r="C214" s="2" t="inlineStr">
+        <is>
+          <t>yes/no</t>
+        </is>
+      </c>
+      <c r="D214" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1011.5 and 1011.6</t>
+        </is>
+      </c>
+      <c r="E214" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F214" s="2" t="n"/>
+      <c r="G214" s="2" t="n"/>
+      <c r="H214" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I214" s="2" t="n"/>
+      <c r="J214" s="2" t="n"/>
+      <c r="K214" s="2" t="n"/>
+      <c r="L214" s="2" t="n"/>
+    </row>
+    <row r="215">
+      <c r="A215" s="2" t="inlineStr">
+        <is>
+          <t>Fire ring, grill or cooking surface</t>
+        </is>
+      </c>
+      <c r="B215" s="2" t="inlineStr">
+        <is>
+          <t>On an access route</t>
+        </is>
+      </c>
+      <c r="C215" s="2" t="inlineStr">
+        <is>
+          <t>yes/no</t>
+        </is>
+      </c>
+      <c r="D215" s="2" t="inlineStr">
+        <is>
+          <t>ABA §F247.1</t>
+        </is>
+      </c>
+      <c r="E215" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F215" s="2" t="n"/>
+      <c r="G215" s="2" t="n"/>
+      <c r="H215" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I215" s="2" t="n"/>
+      <c r="J215" s="2" t="n"/>
+      <c r="K215" s="2" t="n"/>
+      <c r="L215" s="2" t="n"/>
+    </row>
+    <row r="216">
+      <c r="A216" s="2" t="inlineStr">
+        <is>
+          <t>Park bench</t>
+        </is>
+      </c>
+      <c r="B216" s="2" t="inlineStr">
+        <is>
+          <t>Seat height (17 to 19 in)</t>
+        </is>
+      </c>
+      <c r="C216" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D216" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1011.13</t>
+        </is>
+      </c>
+      <c r="E216" s="2" t="inlineStr">
+        <is>
+          <t>min 17, max 19</t>
+        </is>
+      </c>
+      <c r="F216" s="2" t="n"/>
+      <c r="G216" s="2" t="n"/>
+      <c r="H216" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I216" s="2" t="n"/>
+      <c r="J216" s="2" t="n"/>
+      <c r="K216" s="2" t="n"/>
+      <c r="L216" s="2" t="n"/>
+    </row>
+    <row r="217">
+      <c r="A217" s="2" t="inlineStr">
+        <is>
+          <t>Park bench</t>
+        </is>
+      </c>
+      <c r="B217" s="2" t="inlineStr">
+        <is>
+          <t>Back support</t>
+        </is>
+      </c>
+      <c r="C217" s="2" t="inlineStr">
+        <is>
+          <t>yes/no</t>
+        </is>
+      </c>
+      <c r="D217" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1011.13</t>
+        </is>
+      </c>
+      <c r="E217" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F217" s="2" t="n"/>
+      <c r="G217" s="2" t="n"/>
+      <c r="H217" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I217" s="2" t="n"/>
+      <c r="J217" s="2" t="n"/>
+      <c r="K217" s="2" t="n"/>
+      <c r="L217" s="2" t="n"/>
+    </row>
+    <row r="218">
+      <c r="A218" s="2" t="inlineStr">
+        <is>
+          <t>Park bench</t>
+        </is>
+      </c>
+      <c r="B218" s="2" t="inlineStr">
+        <is>
+          <t>Clear ground space beside the bench</t>
+        </is>
+      </c>
+      <c r="C218" s="2" t="inlineStr">
+        <is>
+          <t>yes/no</t>
+        </is>
+      </c>
+      <c r="D218" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1011.13</t>
+        </is>
+      </c>
+      <c r="E218" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F218" s="2" t="n"/>
+      <c r="G218" s="2" t="n"/>
+      <c r="H218" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I218" s="2" t="n"/>
+      <c r="J218" s="2" t="n"/>
+      <c r="K218" s="2" t="n"/>
+      <c r="L218" s="2" t="n"/>
+    </row>
+    <row r="219">
+      <c r="A219" s="2" t="inlineStr">
+        <is>
+          <t>Campsite or tent pad</t>
+        </is>
+      </c>
+      <c r="B219" s="2" t="inlineStr">
+        <is>
+          <t>Firm and stable tent pad</t>
+        </is>
+      </c>
+      <c r="C219" s="2" t="inlineStr">
+        <is>
+          <t>yes/no</t>
+        </is>
+      </c>
+      <c r="D219" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1013.2</t>
+        </is>
+      </c>
+      <c r="E219" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F219" s="2" t="n"/>
+      <c r="G219" s="2" t="n"/>
+      <c r="H219" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I219" s="2" t="n"/>
+      <c r="J219" s="2" t="n"/>
+      <c r="K219" s="2" t="n"/>
+      <c r="L219" s="2" t="n"/>
+    </row>
+    <row r="220">
+      <c r="A220" s="2" t="inlineStr">
+        <is>
+          <t>Campsite or tent pad</t>
+        </is>
+      </c>
+      <c r="B220" s="2" t="inlineStr">
+        <is>
+          <t>Tent pad slope (1:48 max)</t>
+        </is>
+      </c>
+      <c r="C220" s="2" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D220" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1013.3</t>
+        </is>
+      </c>
+      <c r="E220" s="2" t="inlineStr">
+        <is>
+          <t>max 2.08</t>
+        </is>
+      </c>
+      <c r="F220" s="2" t="n"/>
+      <c r="G220" s="2" t="n"/>
+      <c r="H220" s="2" t="inlineStr">
+        <is>
+          <t>1:33 is allowed on surfaces other than asphalt, concrete and boards where needed for drainage. Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I220" s="2" t="n"/>
+      <c r="J220" s="2" t="n"/>
+      <c r="K220" s="2" t="n"/>
+      <c r="L220" s="2" t="n"/>
+    </row>
+    <row r="221">
+      <c r="A221" s="2" t="inlineStr">
+        <is>
+          <t>Campsite or tent pad</t>
+        </is>
+      </c>
+      <c r="B221" s="2" t="inlineStr">
+        <is>
+          <t>Clear ground space around the pad (48 in min)</t>
+        </is>
+      </c>
+      <c r="C221" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D221" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1013.4</t>
+        </is>
+      </c>
+      <c r="E221" s="2" t="inlineStr">
+        <is>
+          <t>min 48</t>
+        </is>
+      </c>
+      <c r="F221" s="2" t="n"/>
+      <c r="G221" s="2" t="n"/>
+      <c r="H221" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I221" s="2" t="n"/>
+      <c r="J221" s="2" t="n"/>
+      <c r="K221" s="2" t="n"/>
+      <c r="L221" s="2" t="n"/>
+    </row>
+    <row r="222">
+      <c r="A222" s="2" t="inlineStr">
+        <is>
+          <t>Campsite or tent pad</t>
+        </is>
+      </c>
+      <c r="B222" s="2" t="inlineStr">
+        <is>
+          <t>On an access route</t>
+        </is>
+      </c>
+      <c r="C222" s="2" t="inlineStr">
+        <is>
+          <t>yes/no</t>
+        </is>
+      </c>
+      <c r="D222" s="2" t="inlineStr">
+        <is>
+          <t>ABA §F244</t>
+        </is>
+      </c>
+      <c r="E222" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F222" s="2" t="n"/>
+      <c r="G222" s="2" t="n"/>
+      <c r="H222" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I222" s="2" t="n"/>
+      <c r="J222" s="2" t="n"/>
+      <c r="K222" s="2" t="n"/>
+      <c r="L222" s="2" t="n"/>
+    </row>
+    <row r="223">
+      <c r="A223" s="2" t="inlineStr">
+        <is>
+          <t>Overlook, viewing area or viewing scope</t>
+        </is>
+      </c>
+      <c r="B223" s="2" t="inlineStr">
+        <is>
+          <t>Clear ground space at viewing spots</t>
+        </is>
+      </c>
+      <c r="C223" s="2" t="inlineStr">
+        <is>
+          <t>yes/no</t>
+        </is>
+      </c>
+      <c r="D223" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1011.14</t>
+        </is>
+      </c>
+      <c r="E223" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F223" s="2" t="n"/>
+      <c r="G223" s="2" t="n"/>
+      <c r="H223" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I223" s="2" t="n"/>
+      <c r="J223" s="2" t="n"/>
+      <c r="K223" s="2" t="n"/>
+      <c r="L223" s="2" t="n"/>
+    </row>
+    <row r="224">
+      <c r="A224" s="2" t="inlineStr">
+        <is>
+          <t>Overlook, viewing area or viewing scope</t>
+        </is>
+      </c>
+      <c r="B224" s="2" t="inlineStr">
+        <is>
+          <t>Clear view at seated eye level</t>
+        </is>
+      </c>
+      <c r="C224" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D224" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1011.14</t>
+        </is>
+      </c>
+      <c r="E224" s="2" t="n"/>
+      <c r="F224" s="2" t="n"/>
+      <c r="G224" s="2" t="n"/>
+      <c r="H224" s="2" t="inlineStr">
+        <is>
+          <t>Check that a seated person can see over or through the railing (about 32 in and above). Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I224" s="2" t="n"/>
+      <c r="J224" s="2" t="n"/>
+      <c r="K224" s="2" t="n"/>
+      <c r="L224" s="2" t="n"/>
+    </row>
+    <row r="225">
+      <c r="A225" s="2" t="inlineStr">
+        <is>
+          <t>Overlook, viewing area or viewing scope</t>
+        </is>
+      </c>
+      <c r="B225" s="2" t="inlineStr">
+        <is>
+          <t>Viewing scope eyepiece (43 to 51 in)</t>
+        </is>
+      </c>
+      <c r="C225" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D225" s="2" t="inlineStr">
+        <is>
+          <t>ABA §1011.15</t>
+        </is>
+      </c>
+      <c r="E225" s="2" t="inlineStr">
+        <is>
+          <t>min 43, max 51</t>
+        </is>
+      </c>
+      <c r="F225" s="2" t="n"/>
+      <c r="G225" s="2" t="n"/>
+      <c r="H225" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I225" s="2" t="n"/>
+      <c r="J225" s="2" t="n"/>
+      <c r="K225" s="2" t="n"/>
+      <c r="L225" s="2" t="n"/>
+    </row>
+    <row r="226">
+      <c r="A226" s="2" t="inlineStr">
+        <is>
+          <t>Overlook, viewing area or viewing scope</t>
+        </is>
+      </c>
+      <c r="B226" s="2" t="inlineStr">
+        <is>
+          <t>On an access route</t>
+        </is>
+      </c>
+      <c r="C226" s="2" t="inlineStr">
+        <is>
+          <t>yes/no</t>
+        </is>
+      </c>
+      <c r="D226" s="2" t="inlineStr">
+        <is>
+          <t>ABA §F246</t>
+        </is>
+      </c>
+      <c r="E226" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F226" s="2" t="n"/>
+      <c r="G226" s="2" t="n"/>
+      <c r="H226" s="2" t="inlineStr">
+        <is>
+          <t>Federal ABA Chapter 10: confirm the section number.</t>
+        </is>
+      </c>
+      <c r="I226" s="2" t="n"/>
+      <c r="J226" s="2" t="n"/>
+      <c r="K226" s="2" t="n"/>
+      <c r="L226" s="2" t="n"/>
+    </row>
+    <row r="227">
+      <c r="A227" s="2" t="inlineStr">
+        <is>
+          <t>Accessible voting station or booth</t>
+        </is>
+      </c>
+      <c r="B227" s="2" t="inlineStr">
+        <is>
+          <t>Route to the station (36 in min)</t>
+        </is>
+      </c>
+      <c r="C227" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D227" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §403.5.1</t>
+        </is>
+      </c>
+      <c r="E227" s="2" t="inlineStr">
+        <is>
+          <t>min 36</t>
+        </is>
+      </c>
+      <c r="F227" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §403.5.1</t>
+        </is>
+      </c>
+      <c r="G227" s="2" t="inlineStr">
+        <is>
+          <t>min 36</t>
+        </is>
+      </c>
+      <c r="H227" s="2" t="n"/>
+      <c r="I227" s="2" t="n"/>
+      <c r="J227" s="2" t="n"/>
+      <c r="K227" s="2" t="n"/>
+      <c r="L227" s="2" t="n"/>
+    </row>
+    <row r="228">
+      <c r="A228" s="2" t="inlineStr">
+        <is>
+          <t>Accessible voting station or booth</t>
+        </is>
+      </c>
+      <c r="B228" s="2" t="inlineStr">
+        <is>
+          <t>Clear floor space</t>
+        </is>
+      </c>
+      <c r="C228" s="2" t="inlineStr">
+        <is>
+          <t>yes/no</t>
+        </is>
+      </c>
+      <c r="D228" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §305.3</t>
+        </is>
+      </c>
+      <c r="E228" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F228" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §305.3</t>
+        </is>
+      </c>
+      <c r="G228" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H228" s="2" t="n"/>
+      <c r="I228" s="2" t="n"/>
+      <c r="J228" s="2" t="n"/>
+      <c r="K228" s="2" t="n"/>
+      <c r="L228" s="2" t="n"/>
+    </row>
+    <row r="229">
+      <c r="A229" s="2" t="inlineStr">
+        <is>
+          <t>Accessible voting station or booth</t>
+        </is>
+      </c>
+      <c r="B229" s="2" t="inlineStr">
+        <is>
+          <t>Surface height (28 to 34 in)</t>
+        </is>
+      </c>
+      <c r="C229" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D229" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §902.3</t>
+        </is>
+      </c>
+      <c r="E229" s="2" t="inlineStr">
+        <is>
+          <t>min 28, max 34</t>
+        </is>
+      </c>
+      <c r="F229" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §902.3</t>
+        </is>
+      </c>
+      <c r="G229" s="2" t="inlineStr">
+        <is>
+          <t>min 28, max 34</t>
+        </is>
+      </c>
+      <c r="H229" s="2" t="n"/>
+      <c r="I229" s="2" t="n"/>
+      <c r="J229" s="2" t="n"/>
+      <c r="K229" s="2" t="n"/>
+      <c r="L229" s="2" t="n"/>
+    </row>
+    <row r="230">
+      <c r="A230" s="2" t="inlineStr">
+        <is>
+          <t>Accessible voting station or booth</t>
+        </is>
+      </c>
+      <c r="B230" s="2" t="inlineStr">
+        <is>
+          <t>Knee clearance (27 in min)</t>
+        </is>
+      </c>
+      <c r="C230" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D230" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §306.3</t>
+        </is>
+      </c>
+      <c r="E230" s="2" t="inlineStr">
+        <is>
+          <t>min 27</t>
+        </is>
+      </c>
+      <c r="F230" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §306.3</t>
+        </is>
+      </c>
+      <c r="G230" s="2" t="inlineStr">
+        <is>
+          <t>min 27</t>
+        </is>
+      </c>
+      <c r="H230" s="2" t="n"/>
+      <c r="I230" s="2" t="n"/>
+      <c r="J230" s="2" t="n"/>
+      <c r="K230" s="2" t="n"/>
+      <c r="L230" s="2" t="n"/>
+    </row>
+    <row r="231">
+      <c r="A231" s="2" t="inlineStr">
+        <is>
+          <t>Accessible voting station or booth</t>
+        </is>
+      </c>
+      <c r="B231" s="2" t="inlineStr">
+        <is>
+          <t>Controls within reach (48 in max)</t>
+        </is>
+      </c>
+      <c r="C231" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D231" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §308.2.1 and 308.3.1</t>
+        </is>
+      </c>
+      <c r="E231" s="2" t="inlineStr">
+        <is>
+          <t>max 48</t>
+        </is>
+      </c>
+      <c r="F231" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §308.2.1 and 308.3.1</t>
+        </is>
+      </c>
+      <c r="G231" s="2" t="inlineStr">
+        <is>
+          <t>max 48</t>
+        </is>
+      </c>
+      <c r="H231" s="2" t="n"/>
+      <c r="I231" s="2" t="n"/>
+      <c r="J231" s="2" t="n"/>
+      <c r="K231" s="2" t="n"/>
+      <c r="L231" s="2" t="n"/>
+    </row>
+    <row r="232">
+      <c r="A232" s="2" t="inlineStr">
+        <is>
+          <t>Accessible voting station or booth</t>
+        </is>
+      </c>
+      <c r="B232" s="2" t="inlineStr">
+        <is>
+          <t>Accessible voting system available</t>
+        </is>
+      </c>
+      <c r="C232" s="2" t="inlineStr">
+        <is>
+          <t>yes/no</t>
+        </is>
+      </c>
+      <c r="D232" s="2" t="inlineStr">
+        <is>
+          <t>Help America Vote Act, 52 U.S.C. §21081(a)(3)</t>
+        </is>
+      </c>
+      <c r="E232" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F232" s="2" t="inlineStr">
+        <is>
+          <t>MCL 168.795a</t>
+        </is>
+      </c>
+      <c r="G232" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H232" s="2" t="n"/>
+      <c r="I232" s="2" t="n"/>
+      <c r="J232" s="2" t="n"/>
+      <c r="K232" s="2" t="n"/>
+      <c r="L232" s="2" t="n"/>
+    </row>
+    <row r="233">
+      <c r="A233" s="2" t="inlineStr">
+        <is>
+          <t>Accessible voting station or booth</t>
+        </is>
+      </c>
+      <c r="B233" s="2" t="inlineStr">
+        <is>
+          <t>Private and independent voting</t>
+        </is>
+      </c>
+      <c r="C233" s="2" t="inlineStr">
+        <is>
+          <t>yes/no</t>
+        </is>
+      </c>
+      <c r="D233" s="2" t="inlineStr">
+        <is>
+          <t>Help America Vote Act, 52 U.S.C. §21081(a)(3)(A); DOJ ADA Checklist for Polling Places</t>
+        </is>
+      </c>
+      <c r="E233" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F233" s="2" t="n"/>
+      <c r="G233" s="2" t="n"/>
+      <c r="H233" s="2" t="n"/>
+      <c r="I233" s="2" t="n"/>
+      <c r="J233" s="2" t="n"/>
+      <c r="K233" s="2" t="n"/>
+      <c r="L233" s="2" t="n"/>
+    </row>
+    <row r="234">
+      <c r="A234" s="2" t="inlineStr">
+        <is>
+          <t>Temporary fix (cones, mat, portable ramp, propped door, bell)</t>
+        </is>
+      </c>
+      <c r="B234" s="2" t="inlineStr">
+        <is>
+          <t>Edge height (1/2 in max, beveled)</t>
+        </is>
+      </c>
+      <c r="C234" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D234" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §303.3</t>
+        </is>
+      </c>
+      <c r="E234" s="2" t="inlineStr">
+        <is>
+          <t>max 0.5</t>
+        </is>
+      </c>
+      <c r="F234" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §303.3</t>
+        </is>
+      </c>
+      <c r="G234" s="2" t="inlineStr">
+        <is>
+          <t>max 0.5</t>
+        </is>
+      </c>
+      <c r="H234" s="2" t="n"/>
+      <c r="I234" s="2" t="n"/>
+      <c r="J234" s="2" t="n"/>
+      <c r="K234" s="2" t="n"/>
+      <c r="L234" s="2" t="n"/>
+    </row>
+    <row r="235">
+      <c r="A235" s="2" t="inlineStr">
+        <is>
+          <t>Temporary fix (cones, mat, portable ramp, propped door, bell)</t>
+        </is>
+      </c>
+      <c r="B235" s="2" t="inlineStr">
+        <is>
+          <t>Portable ramp slope (1:12 max)</t>
+        </is>
+      </c>
+      <c r="C235" s="2" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D235" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §405.2</t>
+        </is>
+      </c>
+      <c r="E235" s="2" t="inlineStr">
+        <is>
+          <t>max 8.33</t>
+        </is>
+      </c>
+      <c r="F235" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §405.2</t>
+        </is>
+      </c>
+      <c r="G235" s="2" t="inlineStr">
+        <is>
+          <t>max 8.33</t>
+        </is>
+      </c>
+      <c r="H235" s="2" t="n"/>
+      <c r="I235" s="2" t="n"/>
+      <c r="J235" s="2" t="n"/>
+      <c r="K235" s="2" t="n"/>
+      <c r="L235" s="2" t="n"/>
+    </row>
+    <row r="236">
+      <c r="A236" s="2" t="inlineStr">
+        <is>
+          <t>Temporary fix (cones, mat, portable ramp, propped door, bell)</t>
+        </is>
+      </c>
+      <c r="B236" s="2" t="inlineStr">
+        <is>
+          <t>Clear width (36 in min)</t>
+        </is>
+      </c>
+      <c r="C236" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D236" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §403.5.1</t>
+        </is>
+      </c>
+      <c r="E236" s="2" t="inlineStr">
+        <is>
+          <t>min 36</t>
+        </is>
+      </c>
+      <c r="F236" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §403.5.1</t>
+        </is>
+      </c>
+      <c r="G236" s="2" t="inlineStr">
+        <is>
+          <t>min 36</t>
+        </is>
+      </c>
+      <c r="H236" s="2" t="n"/>
+      <c r="I236" s="2" t="n"/>
+      <c r="J236" s="2" t="n"/>
+      <c r="K236" s="2" t="n"/>
+      <c r="L236" s="2" t="n"/>
+    </row>
+    <row r="237">
+      <c r="A237" s="2" t="inlineStr">
+        <is>
+          <t>Tent, booth or vendor space</t>
+        </is>
+      </c>
+      <c r="B237" s="2" t="inlineStr">
+        <is>
+          <t>Change in level at the entry</t>
+        </is>
+      </c>
+      <c r="C237" s="2" t="inlineStr">
+        <is>
+          <t>levelChange</t>
+        </is>
+      </c>
+      <c r="D237" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §303.2 and 303.3</t>
+        </is>
+      </c>
+      <c r="E237" s="2" t="n"/>
+      <c r="F237" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §303.2 and 303.3</t>
+        </is>
+      </c>
+      <c r="G237" s="2" t="n"/>
+      <c r="H237" s="2" t="n"/>
+      <c r="I237" s="2" t="n"/>
+      <c r="J237" s="2" t="n"/>
+      <c r="K237" s="2" t="n"/>
+      <c r="L237" s="2" t="n"/>
+    </row>
+    <row r="238">
+      <c r="A238" s="2" t="inlineStr">
+        <is>
+          <t>Tent, booth or vendor space</t>
+        </is>
+      </c>
+      <c r="B238" s="2" t="inlineStr">
+        <is>
+          <t>Entry width (32 in min at openings)</t>
+        </is>
+      </c>
+      <c r="C238" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D238" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §404.2.3</t>
+        </is>
+      </c>
+      <c r="E238" s="2" t="inlineStr">
+        <is>
+          <t>min 32</t>
+        </is>
+      </c>
+      <c r="F238" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §404.2.3</t>
+        </is>
+      </c>
+      <c r="G238" s="2" t="inlineStr">
+        <is>
+          <t>min 32</t>
+        </is>
+      </c>
+      <c r="H238" s="2" t="n"/>
+      <c r="I238" s="2" t="n"/>
+      <c r="J238" s="2" t="n"/>
+      <c r="K238" s="2" t="n"/>
+      <c r="L238" s="2" t="n"/>
+    </row>
+    <row r="239">
+      <c r="A239" s="2" t="inlineStr">
+        <is>
+          <t>Tent, booth or vendor space</t>
+        </is>
+      </c>
+      <c r="B239" s="2" t="inlineStr">
+        <is>
+          <t>Aisle width (36 in min)</t>
+        </is>
+      </c>
+      <c r="C239" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D239" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §403.5.1</t>
+        </is>
+      </c>
+      <c r="E239" s="2" t="inlineStr">
+        <is>
+          <t>min 36</t>
+        </is>
+      </c>
+      <c r="F239" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §403.5.1</t>
+        </is>
+      </c>
+      <c r="G239" s="2" t="inlineStr">
+        <is>
+          <t>min 36</t>
+        </is>
+      </c>
+      <c r="H239" s="2" t="n"/>
+      <c r="I239" s="2" t="n"/>
+      <c r="J239" s="2" t="n"/>
+      <c r="K239" s="2" t="n"/>
+      <c r="L239" s="2" t="n"/>
+    </row>
+    <row r="240">
+      <c r="A240" s="2" t="inlineStr">
+        <is>
+          <t>Tent, booth or vendor space</t>
+        </is>
+      </c>
+      <c r="B240" s="2" t="inlineStr">
+        <is>
+          <t>Turning space</t>
+        </is>
+      </c>
+      <c r="C240" s="2" t="inlineStr">
+        <is>
+          <t>yes/no</t>
+        </is>
+      </c>
+      <c r="D240" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §304.3</t>
+        </is>
+      </c>
+      <c r="E240" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F240" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §304.3</t>
+        </is>
+      </c>
+      <c r="G240" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H240" s="2" t="n"/>
+      <c r="I240" s="2" t="n"/>
+      <c r="J240" s="2" t="n"/>
+      <c r="K240" s="2" t="n"/>
+      <c r="L240" s="2" t="n"/>
+    </row>
+    <row r="241">
+      <c r="A241" s="2" t="inlineStr">
+        <is>
+          <t>Tent, booth or vendor space</t>
+        </is>
+      </c>
+      <c r="B241" s="2" t="inlineStr">
+        <is>
+          <t>Floor surface</t>
+        </is>
+      </c>
+      <c r="C241" s="2" t="inlineStr">
+        <is>
+          <t>yes/no</t>
+        </is>
+      </c>
+      <c r="D241" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §302.1</t>
+        </is>
+      </c>
+      <c r="E241" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F241" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §302.1</t>
+        </is>
+      </c>
+      <c r="G241" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H241" s="2" t="n"/>
+      <c r="I241" s="2" t="n"/>
+      <c r="J241" s="2" t="n"/>
+      <c r="K241" s="2" t="n"/>
+      <c r="L241" s="2" t="n"/>
+    </row>
+    <row r="242">
+      <c r="A242" s="2" t="inlineStr">
+        <is>
+          <t>Tent, booth or vendor space</t>
+        </is>
+      </c>
+      <c r="B242" s="2" t="inlineStr">
+        <is>
+          <t>Service counter or table (36 in max)</t>
+        </is>
+      </c>
+      <c r="C242" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D242" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §904.4.1</t>
+        </is>
+      </c>
+      <c r="E242" s="2" t="inlineStr">
+        <is>
+          <t>max 36</t>
+        </is>
+      </c>
+      <c r="F242" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §904.3.1</t>
+        </is>
+      </c>
+      <c r="G242" s="2" t="inlineStr">
+        <is>
+          <t>max 36</t>
+        </is>
+      </c>
+      <c r="H242" s="2" t="n"/>
+      <c r="I242" s="2" t="n"/>
+      <c r="J242" s="2" t="n"/>
+      <c r="K242" s="2" t="n"/>
+      <c r="L242" s="2" t="n"/>
+    </row>
+    <row r="243">
+      <c r="A243" s="2" t="inlineStr">
+        <is>
+          <t>Tent, booth or vendor space</t>
+        </is>
+      </c>
+      <c r="B243" s="2" t="inlineStr">
+        <is>
+          <t>High reach (48 in max)</t>
+        </is>
+      </c>
+      <c r="C243" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D243" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §308.2.1 and 308.3.1</t>
+        </is>
+      </c>
+      <c r="E243" s="2" t="inlineStr">
+        <is>
+          <t>max 48</t>
+        </is>
+      </c>
+      <c r="F243" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §308.2.1 and 308.3.1</t>
+        </is>
+      </c>
+      <c r="G243" s="2" t="inlineStr">
+        <is>
+          <t>max 48</t>
+        </is>
+      </c>
+      <c r="H243" s="2" t="n"/>
+      <c r="I243" s="2" t="n"/>
+      <c r="J243" s="2" t="n"/>
+      <c r="K243" s="2" t="n"/>
+      <c r="L243" s="2" t="n"/>
+    </row>
+    <row r="244">
+      <c r="A244" s="2" t="inlineStr">
+        <is>
+          <t>Tent, booth or vendor space</t>
+        </is>
+      </c>
+      <c r="B244" s="2" t="inlineStr">
+        <is>
+          <t>Low reach (15 in min)</t>
+        </is>
+      </c>
+      <c r="C244" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D244" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §308.2.1 and 308.3.1</t>
+        </is>
+      </c>
+      <c r="E244" s="2" t="inlineStr">
+        <is>
+          <t>min 15</t>
+        </is>
+      </c>
+      <c r="F244" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §308.2.1 and 308.3.1</t>
+        </is>
+      </c>
+      <c r="G244" s="2" t="inlineStr">
+        <is>
+          <t>min 15</t>
+        </is>
+      </c>
+      <c r="H244" s="2" t="n"/>
+      <c r="I244" s="2" t="n"/>
+      <c r="J244" s="2" t="n"/>
+      <c r="K244" s="2" t="n"/>
+      <c r="L244" s="2" t="n"/>
+    </row>
+    <row r="245">
+      <c r="A245" s="2" t="inlineStr">
+        <is>
+          <t>Event path, ground cover or cable cover</t>
+        </is>
+      </c>
+      <c r="B245" s="2" t="inlineStr">
+        <is>
+          <t>Firm, stable path</t>
+        </is>
+      </c>
+      <c r="C245" s="2" t="inlineStr">
+        <is>
+          <t>yes/no</t>
+        </is>
+      </c>
+      <c r="D245" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §302.1</t>
+        </is>
+      </c>
+      <c r="E245" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F245" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §302.1</t>
+        </is>
+      </c>
+      <c r="G245" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H245" s="2" t="n"/>
+      <c r="I245" s="2" t="n"/>
+      <c r="J245" s="2" t="n"/>
+      <c r="K245" s="2" t="n"/>
+      <c r="L245" s="2" t="n"/>
+    </row>
+    <row r="246">
+      <c r="A246" s="2" t="inlineStr">
+        <is>
+          <t>Event path, ground cover or cable cover</t>
+        </is>
+      </c>
+      <c r="B246" s="2" t="inlineStr">
+        <is>
+          <t>Clear width (36 in min)</t>
+        </is>
+      </c>
+      <c r="C246" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D246" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §403.5.1</t>
+        </is>
+      </c>
+      <c r="E246" s="2" t="inlineStr">
+        <is>
+          <t>min 36</t>
+        </is>
+      </c>
+      <c r="F246" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §403.5.1</t>
+        </is>
+      </c>
+      <c r="G246" s="2" t="inlineStr">
+        <is>
+          <t>min 36</t>
+        </is>
+      </c>
+      <c r="H246" s="2" t="n"/>
+      <c r="I246" s="2" t="n"/>
+      <c r="J246" s="2" t="n"/>
+      <c r="K246" s="2" t="n"/>
+      <c r="L246" s="2" t="n"/>
+    </row>
+    <row r="247">
+      <c r="A247" s="2" t="inlineStr">
+        <is>
+          <t>Event path, ground cover or cable cover</t>
+        </is>
+      </c>
+      <c r="B247" s="2" t="inlineStr">
+        <is>
+          <t>Running slope (1:20 max; steeper needs a ramp)</t>
+        </is>
+      </c>
+      <c r="C247" s="2" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D247" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §403.3</t>
+        </is>
+      </c>
+      <c r="E247" s="2" t="inlineStr">
+        <is>
+          <t>max 5</t>
+        </is>
+      </c>
+      <c r="F247" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §403.3</t>
+        </is>
+      </c>
+      <c r="G247" s="2" t="inlineStr">
+        <is>
+          <t>max 5</t>
+        </is>
+      </c>
+      <c r="H247" s="2" t="n"/>
+      <c r="I247" s="2" t="n"/>
+      <c r="J247" s="2" t="n"/>
+      <c r="K247" s="2" t="n"/>
+      <c r="L247" s="2" t="n"/>
+    </row>
+    <row r="248">
+      <c r="A248" s="2" t="inlineStr">
+        <is>
+          <t>Event path, ground cover or cable cover</t>
+        </is>
+      </c>
+      <c r="B248" s="2" t="inlineStr">
+        <is>
+          <t>Cross slope (1:48 max)</t>
+        </is>
+      </c>
+      <c r="C248" s="2" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D248" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §403.3</t>
+        </is>
+      </c>
+      <c r="E248" s="2" t="inlineStr">
+        <is>
+          <t>max 2.08</t>
+        </is>
+      </c>
+      <c r="F248" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §403.3</t>
+        </is>
+      </c>
+      <c r="G248" s="2" t="inlineStr">
+        <is>
+          <t>max 2.08</t>
+        </is>
+      </c>
+      <c r="H248" s="2" t="n"/>
+      <c r="I248" s="2" t="n"/>
+      <c r="J248" s="2" t="n"/>
+      <c r="K248" s="2" t="n"/>
+      <c r="L248" s="2" t="n"/>
+    </row>
+    <row r="249">
+      <c r="A249" s="2" t="inlineStr">
+        <is>
+          <t>Event path, ground cover or cable cover</t>
+        </is>
+      </c>
+      <c r="B249" s="2" t="inlineStr">
+        <is>
+          <t>Cable covers and edges</t>
+        </is>
+      </c>
+      <c r="C249" s="2" t="inlineStr">
+        <is>
+          <t>levelChange</t>
+        </is>
+      </c>
+      <c r="D249" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §303.2, 303.3 and 303.4</t>
+        </is>
+      </c>
+      <c r="E249" s="2" t="n"/>
+      <c r="F249" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §303.2, 303.3 and 303.4</t>
+        </is>
+      </c>
+      <c r="G249" s="2" t="n"/>
+      <c r="H249" s="2" t="inlineStr">
+        <is>
+          <t>Cable covers over 1/2 in high must have ramped sides (1:12 max).</t>
+        </is>
+      </c>
+      <c r="I249" s="2" t="n"/>
+      <c r="J249" s="2" t="n"/>
+      <c r="K249" s="2" t="n"/>
+      <c r="L249" s="2" t="n"/>
+    </row>
+    <row r="250">
+      <c r="A250" s="2" t="inlineStr">
+        <is>
+          <t>Event path, ground cover or cable cover</t>
+        </is>
+      </c>
+      <c r="B250" s="2" t="inlineStr">
+        <is>
+          <t>Gaps (1/2 in max)</t>
+        </is>
+      </c>
+      <c r="C250" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D250" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §302.3</t>
+        </is>
+      </c>
+      <c r="E250" s="2" t="inlineStr">
+        <is>
+          <t>max 0.5</t>
+        </is>
+      </c>
+      <c r="F250" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §302.3</t>
+        </is>
+      </c>
+      <c r="G250" s="2" t="inlineStr">
+        <is>
+          <t>max 0.5</t>
+        </is>
+      </c>
+      <c r="H250" s="2" t="n"/>
+      <c r="I250" s="2" t="n"/>
+      <c r="J250" s="2" t="n"/>
+      <c r="K250" s="2" t="n"/>
+      <c r="L250" s="2" t="n"/>
+    </row>
+    <row r="251">
+      <c r="A251" s="2" t="inlineStr">
+        <is>
+          <t>Portable toilets</t>
+        </is>
+      </c>
+      <c r="B251" s="2" t="inlineStr">
+        <is>
+          <t>At least 5% accessible (at least one)</t>
+        </is>
+      </c>
+      <c r="C251" s="2" t="inlineStr">
+        <is>
+          <t>ratio</t>
+        </is>
+      </c>
+      <c r="D251" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §213.2</t>
+        </is>
+      </c>
+      <c r="E251" s="2" t="n"/>
+      <c r="F251" s="2" t="inlineStr">
+        <is>
+          <t>2021 MBC §1109.2</t>
+        </is>
+      </c>
+      <c r="G251" s="2" t="n"/>
+      <c r="H251" s="2" t="n"/>
+      <c r="I251" s="2" t="n"/>
+      <c r="J251" s="2" t="n"/>
+      <c r="K251" s="2" t="n"/>
+      <c r="L251" s="2" t="n"/>
+    </row>
+    <row r="252">
+      <c r="A252" s="2" t="inlineStr">
+        <is>
+          <t>Portable toilets</t>
+        </is>
+      </c>
+      <c r="B252" s="2" t="inlineStr">
+        <is>
+          <t>On an accessible route</t>
+        </is>
+      </c>
+      <c r="C252" s="2" t="inlineStr">
+        <is>
+          <t>yes/no</t>
+        </is>
+      </c>
+      <c r="D252" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §206.2.2 and 302.1</t>
+        </is>
+      </c>
+      <c r="E252" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F252" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §302.1</t>
+        </is>
+      </c>
+      <c r="G252" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H252" s="2" t="n"/>
+      <c r="I252" s="2" t="n"/>
+      <c r="J252" s="2" t="n"/>
+      <c r="K252" s="2" t="n"/>
+      <c r="L252" s="2" t="n"/>
+    </row>
+    <row r="253">
+      <c r="A253" s="2" t="inlineStr">
+        <is>
+          <t>Portable toilets</t>
+        </is>
+      </c>
+      <c r="B253" s="2" t="inlineStr">
+        <is>
+          <t>Level entry</t>
+        </is>
+      </c>
+      <c r="C253" s="2" t="inlineStr">
+        <is>
+          <t>levelChange</t>
+        </is>
+      </c>
+      <c r="D253" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §303.2 and 303.3</t>
+        </is>
+      </c>
+      <c r="E253" s="2" t="n"/>
+      <c r="F253" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §303.2 and 303.3</t>
+        </is>
+      </c>
+      <c r="G253" s="2" t="n"/>
+      <c r="H253" s="2" t="n"/>
+      <c r="I253" s="2" t="n"/>
+      <c r="J253" s="2" t="n"/>
+      <c r="K253" s="2" t="n"/>
+      <c r="L253" s="2" t="n"/>
+    </row>
+    <row r="254">
+      <c r="A254" s="2" t="inlineStr">
+        <is>
+          <t>Portable toilets</t>
+        </is>
+      </c>
+      <c r="B254" s="2" t="inlineStr">
+        <is>
+          <t>Door clear width (32 in min)</t>
+        </is>
+      </c>
+      <c r="C254" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D254" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §404.2.3</t>
+        </is>
+      </c>
+      <c r="E254" s="2" t="inlineStr">
+        <is>
+          <t>min 32</t>
+        </is>
+      </c>
+      <c r="F254" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §404.2.3</t>
+        </is>
+      </c>
+      <c r="G254" s="2" t="inlineStr">
+        <is>
+          <t>min 32</t>
+        </is>
+      </c>
+      <c r="H254" s="2" t="n"/>
+      <c r="I254" s="2" t="n"/>
+      <c r="J254" s="2" t="n"/>
+      <c r="K254" s="2" t="n"/>
+      <c r="L254" s="2" t="n"/>
+    </row>
+    <row r="255">
+      <c r="A255" s="2" t="inlineStr">
+        <is>
+          <t>Portable toilets</t>
+        </is>
+      </c>
+      <c r="B255" s="2" t="inlineStr">
+        <is>
+          <t>Turning space inside</t>
+        </is>
+      </c>
+      <c r="C255" s="2" t="inlineStr">
+        <is>
+          <t>yes/no</t>
+        </is>
+      </c>
+      <c r="D255" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §603.2.1</t>
+        </is>
+      </c>
+      <c r="E255" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F255" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §603.2.1</t>
+        </is>
+      </c>
+      <c r="G255" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H255" s="2" t="n"/>
+      <c r="I255" s="2" t="n"/>
+      <c r="J255" s="2" t="n"/>
+      <c r="K255" s="2" t="n"/>
+      <c r="L255" s="2" t="n"/>
+    </row>
+    <row r="256">
+      <c r="A256" s="2" t="inlineStr">
+        <is>
+          <t>Portable toilets</t>
+        </is>
+      </c>
+      <c r="B256" s="2" t="inlineStr">
+        <is>
+          <t>Seat height (17 to 19 in)</t>
+        </is>
+      </c>
+      <c r="C256" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D256" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §604.4</t>
+        </is>
+      </c>
+      <c r="E256" s="2" t="inlineStr">
+        <is>
+          <t>min 17, max 19</t>
+        </is>
+      </c>
+      <c r="F256" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §604.4</t>
+        </is>
+      </c>
+      <c r="G256" s="2" t="inlineStr">
+        <is>
+          <t>min 17, max 19</t>
+        </is>
+      </c>
+      <c r="H256" s="2" t="n"/>
+      <c r="I256" s="2" t="n"/>
+      <c r="J256" s="2" t="n"/>
+      <c r="K256" s="2" t="n"/>
+      <c r="L256" s="2" t="n"/>
+    </row>
+    <row r="257">
+      <c r="A257" s="2" t="inlineStr">
+        <is>
+          <t>Portable toilets</t>
+        </is>
+      </c>
+      <c r="B257" s="2" t="inlineStr">
+        <is>
+          <t>Grab bars</t>
+        </is>
+      </c>
+      <c r="C257" s="2" t="inlineStr">
+        <is>
+          <t>yes/no</t>
+        </is>
+      </c>
+      <c r="D257" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §604.5</t>
+        </is>
+      </c>
+      <c r="E257" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F257" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §604.5</t>
+        </is>
+      </c>
+      <c r="G257" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H257" s="2" t="n"/>
+      <c r="I257" s="2" t="n"/>
+      <c r="J257" s="2" t="n"/>
+      <c r="K257" s="2" t="n"/>
+      <c r="L257" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Check amusement rides, shooting ranges, saunas, EV chargers, lighting and playground safety
Adds six element types that consultants previously had to record as Something else. Rides, shooting ranges and saunas are checked against ADA 2010 and ICC A117.1-2017. EV charging, exterior lighting and playground safety are best-practice or safety items and show as Best practice not met, never as violations. New citations are added to the rules review workbook.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AdurZhc4WrEcjZAJU4UBbC
</commit_message>
<xml_diff>
--- a/Rules review - Michigan citations to verify.xlsx
+++ b/Rules review - Michigan citations to verify.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L257"/>
+  <dimension ref="A1:L296"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -11144,6 +11144,1400 @@
       <c r="K257" s="2" t="n"/>
       <c r="L257" s="2" t="n"/>
     </row>
+    <row r="258">
+      <c r="A258" s="2" t="inlineStr">
+        <is>
+          <t>EV charging station</t>
+        </is>
+      </c>
+      <c r="B258" s="2" t="inlineStr">
+        <is>
+          <t>Accessible EV charging spaces (5% min, at least 1)</t>
+        </is>
+      </c>
+      <c r="C258" s="2" t="inlineStr">
+        <is>
+          <t>ratio</t>
+        </is>
+      </c>
+      <c r="D258" s="2" t="n"/>
+      <c r="E258" s="2" t="n"/>
+      <c r="F258" s="2" t="inlineStr">
+        <is>
+          <t>2021 MBC §1107.2</t>
+        </is>
+      </c>
+      <c r="G258" s="2" t="n"/>
+      <c r="H258" s="2" t="inlineStr">
+        <is>
+          <t>Applies only to work permitted under the 2021 MBC. Applies to chargers installed under the 2021 Michigan Building Code. For older installations the count is shown as best practice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="2" t="inlineStr">
+        <is>
+          <t>EV charging station</t>
+        </is>
+      </c>
+      <c r="B259" s="2" t="inlineStr">
+        <is>
+          <t>Space width (132 in min)</t>
+        </is>
+      </c>
+      <c r="C259" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D259" s="2" t="inlineStr">
+        <is>
+          <t>US Access Board, Design Recommendations for Accessible Electric Vehicle Charging Stations (2023)</t>
+        </is>
+      </c>
+      <c r="E259" s="2" t="inlineStr">
+        <is>
+          <t>min 132</t>
+        </is>
+      </c>
+      <c r="F259" s="2" t="n"/>
+      <c r="G259" s="2" t="n"/>
+      <c r="H259" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Best practice or safety item, not an accessibility requirement. </t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="2" t="inlineStr">
+        <is>
+          <t>EV charging station</t>
+        </is>
+      </c>
+      <c r="B260" s="2" t="inlineStr">
+        <is>
+          <t>Access aisle width (60 in min)</t>
+        </is>
+      </c>
+      <c r="C260" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D260" s="2" t="inlineStr">
+        <is>
+          <t>US Access Board, Design Recommendations for Accessible Electric Vehicle Charging Stations (2023)</t>
+        </is>
+      </c>
+      <c r="E260" s="2" t="inlineStr">
+        <is>
+          <t>min 60</t>
+        </is>
+      </c>
+      <c r="F260" s="2" t="n"/>
+      <c r="G260" s="2" t="n"/>
+      <c r="H260" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Best practice or safety item, not an accessibility requirement. </t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="2" t="inlineStr">
+        <is>
+          <t>EV charging station</t>
+        </is>
+      </c>
+      <c r="B261" s="2" t="inlineStr">
+        <is>
+          <t>Space and aisle slope (1:48 max)</t>
+        </is>
+      </c>
+      <c r="C261" s="2" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D261" s="2" t="inlineStr">
+        <is>
+          <t>US Access Board, Design Recommendations for Accessible Electric Vehicle Charging Stations (2023)</t>
+        </is>
+      </c>
+      <c r="E261" s="2" t="inlineStr">
+        <is>
+          <t>max 2.08</t>
+        </is>
+      </c>
+      <c r="F261" s="2" t="n"/>
+      <c r="G261" s="2" t="n"/>
+      <c r="H261" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Best practice or safety item, not an accessibility requirement. </t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="2" t="inlineStr">
+        <is>
+          <t>EV charging station</t>
+        </is>
+      </c>
+      <c r="B262" s="2" t="inlineStr">
+        <is>
+          <t>On an accessible route</t>
+        </is>
+      </c>
+      <c r="C262" s="2" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="D262" s="2" t="inlineStr">
+        <is>
+          <t>US Access Board, Design Recommendations for Accessible Electric Vehicle Charging Stations (2023)</t>
+        </is>
+      </c>
+      <c r="E262" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F262" s="2" t="n"/>
+      <c r="G262" s="2" t="n"/>
+      <c r="H262" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Best practice or safety item, not an accessibility requirement. </t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="2" t="inlineStr">
+        <is>
+          <t>EV charging station</t>
+        </is>
+      </c>
+      <c r="B263" s="2" t="inlineStr">
+        <is>
+          <t>Clear floor space at the charger</t>
+        </is>
+      </c>
+      <c r="C263" s="2" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="D263" s="2" t="inlineStr">
+        <is>
+          <t>US Access Board, Design Recommendations for Accessible Electric Vehicle Charging Stations (2023)</t>
+        </is>
+      </c>
+      <c r="E263" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F263" s="2" t="n"/>
+      <c r="G263" s="2" t="n"/>
+      <c r="H263" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Best practice or safety item, not an accessibility requirement. </t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="2" t="inlineStr">
+        <is>
+          <t>EV charging station</t>
+        </is>
+      </c>
+      <c r="B264" s="2" t="inlineStr">
+        <is>
+          <t>Highest operable part (48 in max)</t>
+        </is>
+      </c>
+      <c r="C264" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D264" s="2" t="inlineStr">
+        <is>
+          <t>US Access Board, Design Recommendations for Accessible Electric Vehicle Charging Stations (2023); reach range per ADA 308</t>
+        </is>
+      </c>
+      <c r="E264" s="2" t="inlineStr">
+        <is>
+          <t>max 48</t>
+        </is>
+      </c>
+      <c r="F264" s="2" t="n"/>
+      <c r="G264" s="2" t="n"/>
+      <c r="H264" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Best practice or safety item, not an accessibility requirement. </t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="2" t="inlineStr">
+        <is>
+          <t>EV charging station</t>
+        </is>
+      </c>
+      <c r="B265" s="2" t="inlineStr">
+        <is>
+          <t>Lowest operable part (15 in min)</t>
+        </is>
+      </c>
+      <c r="C265" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D265" s="2" t="inlineStr">
+        <is>
+          <t>US Access Board, Design Recommendations for Accessible Electric Vehicle Charging Stations (2023); reach range per ADA 308</t>
+        </is>
+      </c>
+      <c r="E265" s="2" t="inlineStr">
+        <is>
+          <t>min 15</t>
+        </is>
+      </c>
+      <c r="F265" s="2" t="n"/>
+      <c r="G265" s="2" t="n"/>
+      <c r="H265" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Best practice or safety item, not an accessibility requirement. </t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="2" t="inlineStr">
+        <is>
+          <t>EV charging station</t>
+        </is>
+      </c>
+      <c r="B266" s="2" t="inlineStr">
+        <is>
+          <t>Cord reach</t>
+        </is>
+      </c>
+      <c r="C266" s="2" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="D266" s="2" t="inlineStr">
+        <is>
+          <t>US Access Board, Design Recommendations for Accessible Electric Vehicle Charging Stations (2023)</t>
+        </is>
+      </c>
+      <c r="E266" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F266" s="2" t="n"/>
+      <c r="G266" s="2" t="n"/>
+      <c r="H266" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Best practice or safety item, not an accessibility requirement. </t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="2" t="inlineStr">
+        <is>
+          <t>EV charging station</t>
+        </is>
+      </c>
+      <c r="B267" s="2" t="inlineStr">
+        <is>
+          <t>Accessible charging space identified</t>
+        </is>
+      </c>
+      <c r="C267" s="2" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="D267" s="2" t="inlineStr">
+        <is>
+          <t>US Access Board, Design Recommendations for Accessible Electric Vehicle Charging Stations (2023)</t>
+        </is>
+      </c>
+      <c r="E267" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F267" s="2" t="n"/>
+      <c r="G267" s="2" t="n"/>
+      <c r="H267" s="2" t="inlineStr">
+        <is>
+          <t>Best practice or safety item, not an accessibility requirement. The Access Board recommends identifying the space as accessible without reserving it only for placard holders, so the charger is not left unused.</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="2" t="inlineStr">
+        <is>
+          <t>Exterior lighting (route, parking, entrance)</t>
+        </is>
+      </c>
+      <c r="B268" s="2" t="inlineStr">
+        <is>
+          <t>Route lit</t>
+        </is>
+      </c>
+      <c r="C268" s="2" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="D268" s="2" t="inlineStr">
+        <is>
+          <t>Best practice (no ADA or Michigan accessibility rule for exterior lighting)</t>
+        </is>
+      </c>
+      <c r="E268" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F268" s="2" t="n"/>
+      <c r="G268" s="2" t="n"/>
+      <c r="H268" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Best practice or safety item, not an accessibility requirement. </t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="2" t="inlineStr">
+        <is>
+          <t>Exterior lighting (route, parking, entrance)</t>
+        </is>
+      </c>
+      <c r="B269" s="2" t="inlineStr">
+        <is>
+          <t>Accessible parking lit</t>
+        </is>
+      </c>
+      <c r="C269" s="2" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="D269" s="2" t="inlineStr">
+        <is>
+          <t>Best practice (no ADA or Michigan accessibility rule for exterior lighting)</t>
+        </is>
+      </c>
+      <c r="E269" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F269" s="2" t="n"/>
+      <c r="G269" s="2" t="n"/>
+      <c r="H269" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Best practice or safety item, not an accessibility requirement. </t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="2" t="inlineStr">
+        <is>
+          <t>Exterior lighting (route, parking, entrance)</t>
+        </is>
+      </c>
+      <c r="B270" s="2" t="inlineStr">
+        <is>
+          <t>Accessible entrance lit</t>
+        </is>
+      </c>
+      <c r="C270" s="2" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="D270" s="2" t="inlineStr">
+        <is>
+          <t>Best practice (no ADA or Michigan accessibility rule for exterior lighting)</t>
+        </is>
+      </c>
+      <c r="E270" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F270" s="2" t="n"/>
+      <c r="G270" s="2" t="n"/>
+      <c r="H270" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Best practice or safety item, not an accessibility requirement. </t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="2" t="inlineStr">
+        <is>
+          <t>Exterior lighting (route, parking, entrance)</t>
+        </is>
+      </c>
+      <c r="B271" s="2" t="inlineStr">
+        <is>
+          <t>Level changes lit without glare</t>
+        </is>
+      </c>
+      <c r="C271" s="2" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="D271" s="2" t="inlineStr">
+        <is>
+          <t>Best practice (no ADA or Michigan accessibility rule for exterior lighting)</t>
+        </is>
+      </c>
+      <c r="E271" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F271" s="2" t="n"/>
+      <c r="G271" s="2" t="n"/>
+      <c r="H271" s="2" t="inlineStr">
+        <is>
+          <t>Best practice or safety item, not an accessibility requirement. Even light and contrast help people with low vision find steps and curb edges.</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="2" t="inlineStr">
+        <is>
+          <t>Amusement ride</t>
+        </is>
+      </c>
+      <c r="B272" s="2" t="inlineStr">
+        <is>
+          <t>At least one wheelchair space, transfer seat or transfer device</t>
+        </is>
+      </c>
+      <c r="C272" s="2" t="inlineStr">
+        <is>
+          <t>choiceOk</t>
+        </is>
+      </c>
+      <c r="D272" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §234.3</t>
+        </is>
+      </c>
+      <c r="E272" s="2" t="n"/>
+      <c r="F272" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §1102.1</t>
+        </is>
+      </c>
+      <c r="G272" s="2" t="n"/>
+      <c r="H272" s="2" t="n"/>
+    </row>
+    <row r="273">
+      <c r="A273" s="2" t="inlineStr">
+        <is>
+          <t>Amusement ride</t>
+        </is>
+      </c>
+      <c r="B273" s="2" t="inlineStr">
+        <is>
+          <t>Accessible route to load and unload areas</t>
+        </is>
+      </c>
+      <c r="C273" s="2" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="D273" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §206.2.9 and 1002.2</t>
+        </is>
+      </c>
+      <c r="E273" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F273" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §1102.2</t>
+        </is>
+      </c>
+      <c r="G273" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H273" s="2" t="n"/>
+    </row>
+    <row r="274">
+      <c r="A274" s="2" t="inlineStr">
+        <is>
+          <t>Amusement ride</t>
+        </is>
+      </c>
+      <c r="B274" s="2" t="inlineStr">
+        <is>
+          <t>Turning space at load and unload areas</t>
+        </is>
+      </c>
+      <c r="C274" s="2" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="D274" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §1002.3.1</t>
+        </is>
+      </c>
+      <c r="E274" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F274" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §1102.3.1</t>
+        </is>
+      </c>
+      <c r="G274" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H274" s="2" t="n"/>
+    </row>
+    <row r="275">
+      <c r="A275" s="2" t="inlineStr">
+        <is>
+          <t>Amusement ride</t>
+        </is>
+      </c>
+      <c r="B275" s="2" t="inlineStr">
+        <is>
+          <t>Load and unload area slope (1:48 max)</t>
+        </is>
+      </c>
+      <c r="C275" s="2" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D275" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §1002.3.2</t>
+        </is>
+      </c>
+      <c r="E275" s="2" t="inlineStr">
+        <is>
+          <t>max 2.08</t>
+        </is>
+      </c>
+      <c r="F275" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §1102.3.2</t>
+        </is>
+      </c>
+      <c r="G275" s="2" t="inlineStr">
+        <is>
+          <t>max 2.08</t>
+        </is>
+      </c>
+      <c r="H275" s="2" t="n"/>
+    </row>
+    <row r="276">
+      <c r="A276" s="2" t="inlineStr">
+        <is>
+          <t>Amusement ride</t>
+        </is>
+      </c>
+      <c r="B276" s="2" t="inlineStr">
+        <is>
+          <t>Opening into the wheelchair space (32 in min)</t>
+        </is>
+      </c>
+      <c r="C276" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D276" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §1002.4.5</t>
+        </is>
+      </c>
+      <c r="E276" s="2" t="inlineStr">
+        <is>
+          <t>min 32</t>
+        </is>
+      </c>
+      <c r="F276" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §1102.4.5</t>
+        </is>
+      </c>
+      <c r="G276" s="2" t="inlineStr">
+        <is>
+          <t>min 32</t>
+        </is>
+      </c>
+      <c r="H276" s="2" t="n"/>
+    </row>
+    <row r="277">
+      <c r="A277" s="2" t="inlineStr">
+        <is>
+          <t>Amusement ride</t>
+        </is>
+      </c>
+      <c r="B277" s="2" t="inlineStr">
+        <is>
+          <t>Wheelchair space size and slope</t>
+        </is>
+      </c>
+      <c r="C277" s="2" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="D277" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §1002.4.2 and 1002.4.4</t>
+        </is>
+      </c>
+      <c r="E277" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F277" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §1102.4.2 and 1102.4.4</t>
+        </is>
+      </c>
+      <c r="G277" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H277" s="2" t="n"/>
+    </row>
+    <row r="278">
+      <c r="A278" s="2" t="inlineStr">
+        <is>
+          <t>Amusement ride</t>
+        </is>
+      </c>
+      <c r="B278" s="2" t="inlineStr">
+        <is>
+          <t>Companion seat</t>
+        </is>
+      </c>
+      <c r="C278" s="2" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="D278" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §1002.4.7</t>
+        </is>
+      </c>
+      <c r="E278" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F278" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §1102.4.7</t>
+        </is>
+      </c>
+      <c r="G278" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H278" s="2" t="inlineStr">
+        <is>
+          <t>Required where the ride design allows a companion seat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="2" t="inlineStr">
+        <is>
+          <t>Amusement ride</t>
+        </is>
+      </c>
+      <c r="B279" s="2" t="inlineStr">
+        <is>
+          <t>Transfer seat height (14 to 24 in)</t>
+        </is>
+      </c>
+      <c r="C279" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D279" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §1002.5.2</t>
+        </is>
+      </c>
+      <c r="E279" s="2" t="inlineStr">
+        <is>
+          <t>min 14, max 24</t>
+        </is>
+      </c>
+      <c r="F279" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §1102.5.2</t>
+        </is>
+      </c>
+      <c r="G279" s="2" t="inlineStr">
+        <is>
+          <t>min 14, max 24</t>
+        </is>
+      </c>
+      <c r="H279" s="2" t="n"/>
+    </row>
+    <row r="280">
+      <c r="A280" s="2" t="inlineStr">
+        <is>
+          <t>Amusement ride</t>
+        </is>
+      </c>
+      <c r="B280" s="2" t="inlineStr">
+        <is>
+          <t>Signs at queue entrances</t>
+        </is>
+      </c>
+      <c r="C280" s="2" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="D280" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §216.12</t>
+        </is>
+      </c>
+      <c r="E280" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F280" s="2" t="inlineStr">
+        <is>
+          <t>2021 MBC §1111</t>
+        </is>
+      </c>
+      <c r="G280" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H280" s="2" t="n"/>
+    </row>
+    <row r="281">
+      <c r="A281" s="2" t="inlineStr">
+        <is>
+          <t>Shooting range (firing positions)</t>
+        </is>
+      </c>
+      <c r="B281" s="2" t="inlineStr">
+        <is>
+          <t>Accessible firing positions (5% of each type, at least 1)</t>
+        </is>
+      </c>
+      <c r="C281" s="2" t="inlineStr">
+        <is>
+          <t>ratio</t>
+        </is>
+      </c>
+      <c r="D281" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §243</t>
+        </is>
+      </c>
+      <c r="E281" s="2" t="n"/>
+      <c r="F281" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §1110</t>
+        </is>
+      </c>
+      <c r="G281" s="2" t="n"/>
+      <c r="H281" s="2" t="n"/>
+    </row>
+    <row r="282">
+      <c r="A282" s="2" t="inlineStr">
+        <is>
+          <t>Shooting range (firing positions)</t>
+        </is>
+      </c>
+      <c r="B282" s="2" t="inlineStr">
+        <is>
+          <t>On an accessible route</t>
+        </is>
+      </c>
+      <c r="C282" s="2" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="D282" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §206.2.13</t>
+        </is>
+      </c>
+      <c r="E282" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F282" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §1110</t>
+        </is>
+      </c>
+      <c r="G282" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H282" s="2" t="n"/>
+    </row>
+    <row r="283">
+      <c r="A283" s="2" t="inlineStr">
+        <is>
+          <t>Shooting range (firing positions)</t>
+        </is>
+      </c>
+      <c r="B283" s="2" t="inlineStr">
+        <is>
+          <t>Turning space</t>
+        </is>
+      </c>
+      <c r="C283" s="2" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="D283" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §1010.1 and 304.3.1</t>
+        </is>
+      </c>
+      <c r="E283" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F283" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §1110.1</t>
+        </is>
+      </c>
+      <c r="G283" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H283" s="2" t="n"/>
+    </row>
+    <row r="284">
+      <c r="A284" s="2" t="inlineStr">
+        <is>
+          <t>Shooting range (firing positions)</t>
+        </is>
+      </c>
+      <c r="B284" s="2" t="inlineStr">
+        <is>
+          <t>Slope at the position (1:48 max)</t>
+        </is>
+      </c>
+      <c r="C284" s="2" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D284" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §1010.1</t>
+        </is>
+      </c>
+      <c r="E284" s="2" t="inlineStr">
+        <is>
+          <t>max 2.08</t>
+        </is>
+      </c>
+      <c r="F284" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §1110.1</t>
+        </is>
+      </c>
+      <c r="G284" s="2" t="inlineStr">
+        <is>
+          <t>max 2.08</t>
+        </is>
+      </c>
+      <c r="H284" s="2" t="n"/>
+    </row>
+    <row r="285">
+      <c r="A285" s="2" t="inlineStr">
+        <is>
+          <t>Sauna or steam room</t>
+        </is>
+      </c>
+      <c r="B285" s="2" t="inlineStr">
+        <is>
+          <t>Turning space</t>
+        </is>
+      </c>
+      <c r="C285" s="2" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="D285" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §612.3</t>
+        </is>
+      </c>
+      <c r="E285" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F285" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §612.3</t>
+        </is>
+      </c>
+      <c r="G285" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H285" s="2" t="inlineStr">
+        <is>
+          <t>A readily removable bench may overlap the turning space (ADA 612.3 Exception).</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="2" t="inlineStr">
+        <is>
+          <t>Sauna or steam room</t>
+        </is>
+      </c>
+      <c r="B286" s="2" t="inlineStr">
+        <is>
+          <t>Bench length (42 in min)</t>
+        </is>
+      </c>
+      <c r="C286" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D286" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §612.2 and 903.3</t>
+        </is>
+      </c>
+      <c r="E286" s="2" t="inlineStr">
+        <is>
+          <t>min 42</t>
+        </is>
+      </c>
+      <c r="F286" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §612.2 and 903.3</t>
+        </is>
+      </c>
+      <c r="G286" s="2" t="inlineStr">
+        <is>
+          <t>min 42</t>
+        </is>
+      </c>
+      <c r="H286" s="2" t="n"/>
+    </row>
+    <row r="287">
+      <c r="A287" s="2" t="inlineStr">
+        <is>
+          <t>Sauna or steam room</t>
+        </is>
+      </c>
+      <c r="B287" s="2" t="inlineStr">
+        <is>
+          <t>Bench depth (20 to 24 in)</t>
+        </is>
+      </c>
+      <c r="C287" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D287" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §612.2 and 903.3</t>
+        </is>
+      </c>
+      <c r="E287" s="2" t="inlineStr">
+        <is>
+          <t>min 20, max 24</t>
+        </is>
+      </c>
+      <c r="F287" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §612.2 and 903.3</t>
+        </is>
+      </c>
+      <c r="G287" s="2" t="inlineStr">
+        <is>
+          <t>min 20, max 24</t>
+        </is>
+      </c>
+      <c r="H287" s="2" t="n"/>
+    </row>
+    <row r="288">
+      <c r="A288" s="2" t="inlineStr">
+        <is>
+          <t>Sauna or steam room</t>
+        </is>
+      </c>
+      <c r="B288" s="2" t="inlineStr">
+        <is>
+          <t>Bench height (17 to 19 in)</t>
+        </is>
+      </c>
+      <c r="C288" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D288" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §612.2 and 903.5</t>
+        </is>
+      </c>
+      <c r="E288" s="2" t="inlineStr">
+        <is>
+          <t>min 17, max 19</t>
+        </is>
+      </c>
+      <c r="F288" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §612.2 and 903.5</t>
+        </is>
+      </c>
+      <c r="G288" s="2" t="inlineStr">
+        <is>
+          <t>min 17, max 19</t>
+        </is>
+      </c>
+      <c r="H288" s="2" t="n"/>
+    </row>
+    <row r="289">
+      <c r="A289" s="2" t="inlineStr">
+        <is>
+          <t>Sauna or steam room</t>
+        </is>
+      </c>
+      <c r="B289" s="2" t="inlineStr">
+        <is>
+          <t>Back support</t>
+        </is>
+      </c>
+      <c r="C289" s="2" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="D289" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §612.2 and 903.4</t>
+        </is>
+      </c>
+      <c r="E289" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F289" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §612.2 and 903.4</t>
+        </is>
+      </c>
+      <c r="G289" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H289" s="2" t="n"/>
+    </row>
+    <row r="290">
+      <c r="A290" s="2" t="inlineStr">
+        <is>
+          <t>Sauna or steam room</t>
+        </is>
+      </c>
+      <c r="B290" s="2" t="inlineStr">
+        <is>
+          <t>Clear floor space at the bench</t>
+        </is>
+      </c>
+      <c r="C290" s="2" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="D290" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §612.2 and 903.2</t>
+        </is>
+      </c>
+      <c r="E290" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F290" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §612.2 and 903.2</t>
+        </is>
+      </c>
+      <c r="G290" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H290" s="2" t="n"/>
+    </row>
+    <row r="291">
+      <c r="A291" s="2" t="inlineStr">
+        <is>
+          <t>Sauna or steam room</t>
+        </is>
+      </c>
+      <c r="B291" s="2" t="inlineStr">
+        <is>
+          <t>Door does not swing into the bench clear floor space</t>
+        </is>
+      </c>
+      <c r="C291" s="2" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="D291" s="2" t="inlineStr">
+        <is>
+          <t>ADA 2010 §612.2</t>
+        </is>
+      </c>
+      <c r="E291" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F291" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §612.2</t>
+        </is>
+      </c>
+      <c r="G291" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H291" s="2" t="n"/>
+    </row>
+    <row r="292">
+      <c r="A292" s="2" t="inlineStr">
+        <is>
+          <t>Playground safety check (not accessibility)</t>
+        </is>
+      </c>
+      <c r="B292" s="2" t="inlineStr">
+        <is>
+          <t>Protective surfacing</t>
+        </is>
+      </c>
+      <c r="C292" s="2" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="D292" s="2" t="inlineStr">
+        <is>
+          <t>CPSC Public Playground Safety Handbook, adopted by Michigan's Playground Equipment Safety Act (1997 PA 16)</t>
+        </is>
+      </c>
+      <c r="E292" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F292" s="2" t="n"/>
+      <c r="G292" s="2" t="n"/>
+      <c r="H292" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Best practice or safety item, not an accessibility requirement. </t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="2" t="inlineStr">
+        <is>
+          <t>Playground safety check (not accessibility)</t>
+        </is>
+      </c>
+      <c r="B293" s="2" t="inlineStr">
+        <is>
+          <t>Use zones clear (6 ft min)</t>
+        </is>
+      </c>
+      <c r="C293" s="2" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="D293" s="2" t="inlineStr">
+        <is>
+          <t>CPSC Public Playground Safety Handbook, adopted by Michigan's Playground Equipment Safety Act (1997 PA 16)</t>
+        </is>
+      </c>
+      <c r="E293" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F293" s="2" t="n"/>
+      <c r="G293" s="2" t="n"/>
+      <c r="H293" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Best practice or safety item, not an accessibility requirement. </t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="2" t="inlineStr">
+        <is>
+          <t>Playground safety check (not accessibility)</t>
+        </is>
+      </c>
+      <c r="B294" s="2" t="inlineStr">
+        <is>
+          <t>No head entrapment openings</t>
+        </is>
+      </c>
+      <c r="C294" s="2" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="D294" s="2" t="inlineStr">
+        <is>
+          <t>CPSC Public Playground Safety Handbook, adopted by Michigan's Playground Equipment Safety Act (1997 PA 16)</t>
+        </is>
+      </c>
+      <c r="E294" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F294" s="2" t="n"/>
+      <c r="G294" s="2" t="n"/>
+      <c r="H294" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Best practice or safety item, not an accessibility requirement. </t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="2" t="inlineStr">
+        <is>
+          <t>Playground safety check (not accessibility)</t>
+        </is>
+      </c>
+      <c r="B295" s="2" t="inlineStr">
+        <is>
+          <t>Equipment in good repair</t>
+        </is>
+      </c>
+      <c r="C295" s="2" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="D295" s="2" t="inlineStr">
+        <is>
+          <t>CPSC Public Playground Safety Handbook, adopted by Michigan's Playground Equipment Safety Act (1997 PA 16)</t>
+        </is>
+      </c>
+      <c r="E295" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F295" s="2" t="n"/>
+      <c r="G295" s="2" t="n"/>
+      <c r="H295" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Best practice or safety item, not an accessibility requirement. </t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="2" t="inlineStr">
+        <is>
+          <t>Playground safety check (not accessibility)</t>
+        </is>
+      </c>
+      <c r="B296" s="2" t="inlineStr">
+        <is>
+          <t>Inspection record</t>
+        </is>
+      </c>
+      <c r="C296" s="2" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="D296" s="2" t="inlineStr">
+        <is>
+          <t>CPSC Public Playground Safety Handbook, adopted by Michigan's Playground Equipment Safety Act (1997 PA 16)</t>
+        </is>
+      </c>
+      <c r="E296" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F296" s="2" t="n"/>
+      <c r="G296" s="2" t="n"/>
+      <c r="H296" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Best practice or safety item, not an accessibility requirement. </t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Correct A117.1-2017 recreation section numbers and confirm new ADA citations
ICC A117.1-2017 puts recreational facilities in Chapter 10, with the same section numbers as the 2010 ADA Standards, so every Michigan recreation citation moves from 11xx to 10xx. Boating route scoping is ADA 206.2.10, not 206.2.14. Ride citations confirmed against the Access Board text lose their dagger. The 2021 IBC 1107.2 EV space and aisle sizes are now code requirements for new installs.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AdurZhc4WrEcjZAJU4UBbC
</commit_message>
<xml_diff>
--- a/Rules review - Michigan citations to verify.xlsx
+++ b/Rules review - Michigan citations to verify.xlsx
@@ -5512,11 +5512,15 @@
       <c r="E120" s="2" t="n"/>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1108 (play areas)</t>
+          <t>ICC A117.1-2017 §1008 (play areas)</t>
         </is>
       </c>
       <c r="G120" s="2" t="n"/>
-      <c r="H120" s="2" t="n"/>
+      <c r="H120" s="2" t="inlineStr">
+        <is>
+          <t>Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
+        </is>
+      </c>
       <c r="I120" s="2" t="n"/>
       <c r="J120" s="2" t="n"/>
       <c r="K120" s="2" t="n"/>
@@ -5546,11 +5550,15 @@
       <c r="E121" s="2" t="n"/>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1108 (play areas)</t>
+          <t>ICC A117.1-2017 §1008 (play areas)</t>
         </is>
       </c>
       <c r="G121" s="2" t="n"/>
-      <c r="H121" s="2" t="n"/>
+      <c r="H121" s="2" t="inlineStr">
+        <is>
+          <t>Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
+        </is>
+      </c>
       <c r="I121" s="2" t="n"/>
       <c r="J121" s="2" t="n"/>
       <c r="K121" s="2" t="n"/>
@@ -5580,13 +5588,13 @@
       <c r="E122" s="2" t="n"/>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1108 (play areas)</t>
+          <t>ICC A117.1-2017 §1008 (play areas)</t>
         </is>
       </c>
       <c r="G122" s="2" t="n"/>
       <c r="H122" s="2" t="inlineStr">
         <is>
-          <t>At least one of each type of ground-level component must be on a route; Table 240.2.1.2 adds more based on the number of elevated components. Compare with the counts recorded.</t>
+          <t>At least one of each type of ground-level component must be on a route; Table 240.2.1.2 adds more based on the number of elevated components. Compare with the counts recorded. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I122" s="2" t="n"/>
@@ -5622,7 +5630,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1108.2.4.1</t>
+          <t>ICC A117.1-2017 §1008.2.4.1</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -5632,7 +5640,7 @@
       </c>
       <c r="H123" s="2" t="inlineStr">
         <is>
-          <t>May narrow to 36 in for 60 in max length in play areas under 1,000 sq ft, with conditions (ADA 1008.2.4.1 Exceptions). Also confirm the ADA 2010 sub-section number.</t>
+          <t>May narrow to 36 in for 60 in max length in play areas under 1,000 sq ft, with conditions (ADA 1008.2.4.1 Exceptions). Also confirm the ADA 2010 sub-section number. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I123" s="2" t="n"/>
@@ -5668,7 +5676,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1108.2.6.1</t>
+          <t>ICC A117.1-2017 §1008.2.6.1</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -5676,7 +5684,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H124" s="2" t="n"/>
+      <c r="H124" s="2" t="inlineStr">
+        <is>
+          <t>Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
+        </is>
+      </c>
       <c r="I124" s="2" t="n"/>
       <c r="J124" s="2" t="n"/>
       <c r="K124" s="2" t="n"/>
@@ -5710,7 +5722,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1108.2.6.2</t>
+          <t>ICC A117.1-2017 §1008.2.6.2</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -5718,7 +5730,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H125" s="2" t="n"/>
+      <c r="H125" s="2" t="inlineStr">
+        <is>
+          <t>Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
+        </is>
+      </c>
       <c r="I125" s="2" t="n"/>
       <c r="J125" s="2" t="n"/>
       <c r="K125" s="2" t="n"/>
@@ -5752,7 +5768,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1108.4.1</t>
+          <t>ICC A117.1-2017 §1008.4.1</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -5762,7 +5778,7 @@
       </c>
       <c r="H126" s="2" t="inlineStr">
         <is>
-          <t>Also confirm the ADA 2010 sub-section number.</t>
+          <t>Also confirm the ADA 2010 sub-section number. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I126" s="2" t="n"/>
@@ -5798,7 +5814,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1108.2.5.1</t>
+          <t>ICC A117.1-2017 §1008.2.5.1</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -5808,7 +5824,7 @@
       </c>
       <c r="H127" s="2" t="inlineStr">
         <is>
-          <t>Also confirm the ADA 2010 sub-section number.</t>
+          <t>Also confirm the ADA 2010 sub-section number. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I127" s="2" t="n"/>
@@ -5844,7 +5860,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1108.2.5 and 405.2</t>
+          <t>ICC A117.1-2017 §1008.2.5 and 405.2</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -5854,7 +5870,7 @@
       </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
-          <t>Also confirm the ADA 2010 sub-section number.</t>
+          <t>Also confirm the ADA 2010 sub-section number. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I128" s="2" t="n"/>
@@ -5890,7 +5906,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1108.2.5.2</t>
+          <t>ICC A117.1-2017 §1008.2.5.2</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -5900,7 +5916,7 @@
       </c>
       <c r="H129" s="2" t="inlineStr">
         <is>
-          <t>Also confirm the ADA 2010 sub-section number.</t>
+          <t>Also confirm the ADA 2010 sub-section number. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I129" s="2" t="n"/>
@@ -5936,7 +5952,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1108.2.4.2</t>
+          <t>ICC A117.1-2017 §1008.2.4.2</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -5946,7 +5962,7 @@
       </c>
       <c r="H130" s="2" t="inlineStr">
         <is>
-          <t>Also confirm the ADA 2010 sub-section number.</t>
+          <t>Also confirm the ADA 2010 sub-section number. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I130" s="2" t="n"/>
@@ -5982,7 +5998,7 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1108.2.4.1</t>
+          <t>ICC A117.1-2017 §1008.2.4.1</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
@@ -5992,7 +6008,7 @@
       </c>
       <c r="H131" s="2" t="inlineStr">
         <is>
-          <t>Also confirm the ADA 2010 sub-section number.</t>
+          <t>Also confirm the ADA 2010 sub-section number. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I131" s="2" t="n"/>
@@ -6028,7 +6044,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1108.2.5.3</t>
+          <t>ICC A117.1-2017 §1008.2.5.3</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -6038,7 +6054,7 @@
       </c>
       <c r="H132" s="2" t="inlineStr">
         <is>
-          <t>Handrails are not required on ramps inside ground-level use zones (ADA 1008.2.5.3 Exception). Also confirm the ADA 2010 sub-section number.</t>
+          <t>Handrails are not required on ramps inside ground-level use zones (ADA 1008.2.5.3 Exception). Also confirm the ADA 2010 sub-section number. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I132" s="2" t="n"/>
@@ -6074,7 +6090,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1108.3.1.1</t>
+          <t>ICC A117.1-2017 §1008.3.1.1</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -6084,7 +6100,7 @@
       </c>
       <c r="H133" s="2" t="inlineStr">
         <is>
-          <t>Also confirm the ADA 2010 sub-section number.</t>
+          <t>Also confirm the ADA 2010 sub-section number. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I133" s="2" t="n"/>
@@ -6120,7 +6136,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1108.3.2.1</t>
+          <t>ICC A117.1-2017 §1008.3.2.1</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -6130,7 +6146,7 @@
       </c>
       <c r="H134" s="2" t="inlineStr">
         <is>
-          <t>Also confirm the ADA 2010 sub-section number.</t>
+          <t>Also confirm the ADA 2010 sub-section number. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I134" s="2" t="n"/>
@@ -6166,7 +6182,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1108.3.1.2 and 1108.3.2.2</t>
+          <t>ICC A117.1-2017 §1008.3.1.2 and 1008.3.2.2</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -6176,7 +6192,7 @@
       </c>
       <c r="H135" s="2" t="inlineStr">
         <is>
-          <t>Also confirm the ADA 2010 sub-section number.</t>
+          <t>Also confirm the ADA 2010 sub-section number. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I135" s="2" t="n"/>
@@ -6212,7 +6228,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1108.3.1.2 and 1108.3.2.2</t>
+          <t>ICC A117.1-2017 §1008.3.1.2 and 1008.3.2.2</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -6222,7 +6238,7 @@
       </c>
       <c r="H136" s="2" t="inlineStr">
         <is>
-          <t>Also confirm the ADA 2010 sub-section number.</t>
+          <t>Also confirm the ADA 2010 sub-section number. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I136" s="2" t="n"/>
@@ -6258,7 +6274,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1108.3.1.4 and 1108.3.2.3</t>
+          <t>ICC A117.1-2017 §1008.3.1.4 and 1008.3.2.3</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -6268,7 +6284,7 @@
       </c>
       <c r="H137" s="2" t="inlineStr">
         <is>
-          <t>Also confirm the ADA 2010 sub-section number.</t>
+          <t>Also confirm the ADA 2010 sub-section number. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I137" s="2" t="n"/>
@@ -6304,7 +6320,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1108.2</t>
+          <t>ICC A117.1-2017 §1008.2</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -6312,7 +6328,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H138" s="2" t="n"/>
+      <c r="H138" s="2" t="inlineStr">
+        <is>
+          <t>Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
+        </is>
+      </c>
       <c r="I138" s="2" t="n"/>
       <c r="J138" s="2" t="n"/>
       <c r="K138" s="2" t="n"/>
@@ -6346,7 +6366,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1108.4.2</t>
+          <t>ICC A117.1-2017 §1008.4.2</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -6356,7 +6376,7 @@
       </c>
       <c r="H139" s="2" t="inlineStr">
         <is>
-          <t>Also confirm the ADA 2010 sub-section number.</t>
+          <t>Also confirm the ADA 2010 sub-section number. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I139" s="2" t="n"/>
@@ -6392,7 +6412,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1108.4.4</t>
+          <t>ICC A117.1-2017 §1008.4.4</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -6402,7 +6422,7 @@
       </c>
       <c r="H140" s="2" t="inlineStr">
         <is>
-          <t>Also confirm the ADA 2010 sub-section number.</t>
+          <t>Also confirm the ADA 2010 sub-section number. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I140" s="2" t="n"/>
@@ -6438,7 +6458,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1108.4.3</t>
+          <t>ICC A117.1-2017 §1008.4.3</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -6448,7 +6468,7 @@
       </c>
       <c r="H141" s="2" t="inlineStr">
         <is>
-          <t>Also confirm the ADA 2010 sub-section number.</t>
+          <t>Also confirm the ADA 2010 sub-section number. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I141" s="2" t="n"/>
@@ -6484,7 +6504,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1108.4.3</t>
+          <t>ICC A117.1-2017 §1008.4.3</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -6494,7 +6514,7 @@
       </c>
       <c r="H142" s="2" t="inlineStr">
         <is>
-          <t>Tables for children under 5 may use a parallel approach instead of knee clearance (ADA 1008.4.3 Exception). Also confirm the ADA 2010 sub-section number.</t>
+          <t>Tables for children under 5 may use a parallel approach instead of knee clearance (ADA 1008.4.3 Exception). Also confirm the ADA 2010 sub-section number. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I142" s="2" t="n"/>
@@ -6526,11 +6546,15 @@
       <c r="E143" s="2" t="n"/>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2021 MBC §1110 (pools); ICC A117.1-2017 §1109</t>
+          <t>2021 MBC §1110 (pools); ICC A117.1-2017 §1009</t>
         </is>
       </c>
       <c r="G143" s="2" t="n"/>
-      <c r="H143" s="2" t="n"/>
+      <c r="H143" s="2" t="inlineStr">
+        <is>
+          <t>Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
+        </is>
+      </c>
       <c r="I143" s="2" t="n"/>
       <c r="J143" s="2" t="n"/>
       <c r="K143" s="2" t="n"/>
@@ -6564,7 +6588,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2021 MBC §1110; ICC A117.1-2017 §1109</t>
+          <t>2021 MBC §1110; ICC A117.1-2017 §1009</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -6572,7 +6596,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H144" s="2" t="n"/>
+      <c r="H144" s="2" t="inlineStr">
+        <is>
+          <t>Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
+        </is>
+      </c>
       <c r="I144" s="2" t="n"/>
       <c r="J144" s="2" t="n"/>
       <c r="K144" s="2" t="n"/>
@@ -6606,7 +6634,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1109.2.1</t>
+          <t>ICC A117.1-2017 §1009.2.1</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -6616,7 +6644,7 @@
       </c>
       <c r="H145" s="2" t="inlineStr">
         <is>
-          <t>Exception where the entire pool is deeper than 48 in.</t>
+          <t>Exception where the entire pool is deeper than 48 in. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I145" s="2" t="n"/>
@@ -6652,7 +6680,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1109.2.3</t>
+          <t>ICC A117.1-2017 §1009.2.3</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -6662,7 +6690,7 @@
       </c>
       <c r="H146" s="2" t="inlineStr">
         <is>
-          <t>Also confirm the ADA 2010 sub-section number.</t>
+          <t>Also confirm the ADA 2010 sub-section number. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I146" s="2" t="n"/>
@@ -6698,7 +6726,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1109.2.4</t>
+          <t>ICC A117.1-2017 §1009.2.4</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -6708,7 +6736,7 @@
       </c>
       <c r="H147" s="2" t="inlineStr">
         <is>
-          <t>Also confirm the ADA 2010 sub-section number.</t>
+          <t>Also confirm the ADA 2010 sub-section number. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I147" s="2" t="n"/>
@@ -6744,7 +6772,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1109.2.8</t>
+          <t>ICC A117.1-2017 §1009.2.8</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -6754,7 +6782,7 @@
       </c>
       <c r="H148" s="2" t="inlineStr">
         <is>
-          <t>Also confirm the ADA 2010 sub-section number.</t>
+          <t>Also confirm the ADA 2010 sub-section number. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I148" s="2" t="n"/>
@@ -6790,7 +6818,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1109.2.5</t>
+          <t>ICC A117.1-2017 §1009.2.5</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -6800,7 +6828,7 @@
       </c>
       <c r="H149" s="2" t="inlineStr">
         <is>
-          <t>Also confirm the ADA 2010 sub-section number.</t>
+          <t>Also confirm the ADA 2010 sub-section number. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I149" s="2" t="n"/>
@@ -6836,7 +6864,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1109.2.7</t>
+          <t>ICC A117.1-2017 §1009.2.7</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -6846,7 +6874,7 @@
       </c>
       <c r="H150" s="2" t="inlineStr">
         <is>
-          <t>Also confirm the ADA 2010 sub-section number.</t>
+          <t>Also confirm the ADA 2010 sub-section number. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I150" s="2" t="n"/>
@@ -6882,7 +6910,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1109.2.9</t>
+          <t>ICC A117.1-2017 §1009.2.9</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
@@ -6892,7 +6920,7 @@
       </c>
       <c r="H151" s="2" t="inlineStr">
         <is>
-          <t>Also confirm the ADA 2010 sub-section number.</t>
+          <t>Also confirm the ADA 2010 sub-section number. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I151" s="2" t="n"/>
@@ -6928,7 +6956,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1109.2.2</t>
+          <t>ICC A117.1-2017 §1009.2.2</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -6938,7 +6966,7 @@
       </c>
       <c r="H152" s="2" t="inlineStr">
         <is>
-          <t>Also confirm the ADA 2010 sub-section number.</t>
+          <t>Also confirm the ADA 2010 sub-section number. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I152" s="2" t="n"/>
@@ -6974,7 +7002,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1109.3.1 and 405.2</t>
+          <t>ICC A117.1-2017 §1009.3.1 and 405.2</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -6984,7 +7012,7 @@
       </c>
       <c r="H153" s="2" t="inlineStr">
         <is>
-          <t>Also confirm the ADA 2010 sub-section number.</t>
+          <t>Also confirm the ADA 2010 sub-section number. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I153" s="2" t="n"/>
@@ -7020,7 +7048,7 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1109.3.2</t>
+          <t>ICC A117.1-2017 §1009.3.2</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
@@ -7030,7 +7058,7 @@
       </c>
       <c r="H154" s="2" t="inlineStr">
         <is>
-          <t>Also confirm the ADA 2010 sub-section number.</t>
+          <t>Also confirm the ADA 2010 sub-section number. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I154" s="2" t="n"/>
@@ -7066,7 +7094,7 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1109.3.3</t>
+          <t>ICC A117.1-2017 §1009.3.3</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
@@ -7076,7 +7104,7 @@
       </c>
       <c r="H155" s="2" t="inlineStr">
         <is>
-          <t>Also confirm the ADA 2010 sub-section number.</t>
+          <t>Also confirm the ADA 2010 sub-section number. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I155" s="2" t="n"/>
@@ -7112,7 +7140,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1109.4.2</t>
+          <t>ICC A117.1-2017 §1009.4.2</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -7122,7 +7150,7 @@
       </c>
       <c r="H156" s="2" t="inlineStr">
         <is>
-          <t>Also confirm the ADA 2010 sub-section number.</t>
+          <t>Also confirm the ADA 2010 sub-section number. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I156" s="2" t="n"/>
@@ -7158,7 +7186,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1109.4.3</t>
+          <t>ICC A117.1-2017 §1009.4.3</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
@@ -7168,7 +7196,7 @@
       </c>
       <c r="H157" s="2" t="inlineStr">
         <is>
-          <t>Also confirm the ADA 2010 sub-section number.</t>
+          <t>Also confirm the ADA 2010 sub-section number. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I157" s="2" t="n"/>
@@ -7204,7 +7232,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1109.4.3</t>
+          <t>ICC A117.1-2017 §1009.4.3</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
@@ -7214,7 +7242,7 @@
       </c>
       <c r="H158" s="2" t="inlineStr">
         <is>
-          <t>Also confirm the ADA 2010 sub-section number.</t>
+          <t>Also confirm the ADA 2010 sub-section number. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I158" s="2" t="n"/>
@@ -7250,7 +7278,7 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1109.4.5</t>
+          <t>ICC A117.1-2017 §1009.4.5</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
@@ -7260,7 +7288,7 @@
       </c>
       <c r="H159" s="2" t="inlineStr">
         <is>
-          <t>Also confirm the ADA 2010 sub-section number.</t>
+          <t>Also confirm the ADA 2010 sub-section number. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I159" s="2" t="n"/>
@@ -7540,7 +7568,7 @@
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1105.2.1</t>
+          <t>ICC A117.1-2017 §1005.2.1</t>
         </is>
       </c>
       <c r="G166" s="2" t="inlineStr">
@@ -7548,7 +7576,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H166" s="2" t="n"/>
+      <c r="H166" s="2" t="inlineStr">
+        <is>
+          <t>Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
+        </is>
+      </c>
       <c r="I166" s="2" t="n"/>
       <c r="J166" s="2" t="n"/>
       <c r="K166" s="2" t="n"/>
@@ -7582,7 +7614,7 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1105.2.2</t>
+          <t>ICC A117.1-2017 §1005.2.2</t>
         </is>
       </c>
       <c r="G167" s="2" t="inlineStr">
@@ -7592,7 +7624,7 @@
       </c>
       <c r="H167" s="2" t="inlineStr">
         <is>
-          <t>Also confirm the ADA 2010 sub-section number.</t>
+          <t>Also confirm the ADA 2010 sub-section number. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I167" s="2" t="n"/>
@@ -7628,7 +7660,7 @@
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1105.3</t>
+          <t>ICC A117.1-2017 §1005.3</t>
         </is>
       </c>
       <c r="G168" s="2" t="inlineStr">
@@ -7636,7 +7668,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H168" s="2" t="n"/>
+      <c r="H168" s="2" t="inlineStr">
+        <is>
+          <t>Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
+        </is>
+      </c>
       <c r="I168" s="2" t="n"/>
       <c r="J168" s="2" t="n"/>
       <c r="K168" s="2" t="n"/>
@@ -7670,7 +7706,7 @@
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1105.4</t>
+          <t>ICC A117.1-2017 §1005.4</t>
         </is>
       </c>
       <c r="G169" s="2" t="inlineStr">
@@ -7678,7 +7714,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H169" s="2" t="n"/>
+      <c r="H169" s="2" t="inlineStr">
+        <is>
+          <t>Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
+        </is>
+      </c>
       <c r="I169" s="2" t="n"/>
       <c r="J169" s="2" t="n"/>
       <c r="K169" s="2" t="n"/>
@@ -7712,7 +7752,7 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1103.2.1</t>
+          <t>ICC A117.1-2017 §1003.2.1</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
@@ -7722,7 +7762,7 @@
       </c>
       <c r="H170" s="2" t="inlineStr">
         <is>
-          <t>Longer gangways and tidal or changing water levels have exceptions (ADA 1003.2.1 Exceptions); check them before reporting a failure. Also confirm the ADA 2010 sub-section number.</t>
+          <t>Longer gangways and tidal or changing water levels have exceptions (ADA 1003.2.1 Exceptions); check them before reporting a failure. Also confirm the ADA 2010 sub-section number. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I170" s="2" t="n"/>
@@ -7758,7 +7798,7 @@
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1103.3.1</t>
+          <t>ICC A117.1-2017 §1003.3.1</t>
         </is>
       </c>
       <c r="G171" s="2" t="inlineStr">
@@ -7768,7 +7808,7 @@
       </c>
       <c r="H171" s="2" t="inlineStr">
         <is>
-          <t>Also confirm the ADA 2010 sub-section number.</t>
+          <t>Also confirm the ADA 2010 sub-section number. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I171" s="2" t="n"/>
@@ -7794,7 +7834,7 @@
       </c>
       <c r="D172" s="2" t="inlineStr">
         <is>
-          <t>ADA 2010 §206.2.14 and 1003.2</t>
+          <t>ADA 2010 §206.2.10 and 1003.2</t>
         </is>
       </c>
       <c r="E172" s="2" t="inlineStr">
@@ -7804,7 +7844,7 @@
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1103.2</t>
+          <t>ICC A117.1-2017 §1003.2</t>
         </is>
       </c>
       <c r="G172" s="2" t="inlineStr">
@@ -7814,7 +7854,7 @@
       </c>
       <c r="H172" s="2" t="inlineStr">
         <is>
-          <t>Also confirm the ADA 2010 sub-section number.</t>
+          <t>Also confirm the ADA 2010 sub-section number. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I172" s="2" t="n"/>
@@ -7850,7 +7890,7 @@
       </c>
       <c r="F173" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1106.3.2</t>
+          <t>ICC A117.1-2017 §1006.3.2</t>
         </is>
       </c>
       <c r="G173" s="2" t="inlineStr">
@@ -7860,7 +7900,7 @@
       </c>
       <c r="H173" s="2" t="inlineStr">
         <is>
-          <t>Also confirm the ADA 2010 sub-section number.</t>
+          <t>Also confirm the ADA 2010 sub-section number. Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
         </is>
       </c>
       <c r="I173" s="2" t="n"/>
@@ -7892,11 +7932,15 @@
       <c r="E174" s="2" t="n"/>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1107.2</t>
+          <t>ICC A117.1-2017 §1007.2</t>
         </is>
       </c>
       <c r="G174" s="2" t="n"/>
-      <c r="H174" s="2" t="n"/>
+      <c r="H174" s="2" t="inlineStr">
+        <is>
+          <t>Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
+        </is>
+      </c>
       <c r="I174" s="2" t="n"/>
       <c r="J174" s="2" t="n"/>
       <c r="K174" s="2" t="n"/>
@@ -7930,7 +7974,7 @@
       </c>
       <c r="F175" s="2" t="inlineStr">
         <is>
-          <t>2021 MBC §1110; ICC A117.1-2017 §1104</t>
+          <t>2021 MBC §1110; ICC A117.1-2017 §1004</t>
         </is>
       </c>
       <c r="G175" s="2" t="inlineStr">
@@ -7938,7 +7982,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H175" s="2" t="n"/>
+      <c r="H175" s="2" t="inlineStr">
+        <is>
+          <t>Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
+        </is>
+      </c>
       <c r="I175" s="2" t="n"/>
       <c r="J175" s="2" t="n"/>
       <c r="K175" s="2" t="n"/>
@@ -7972,7 +8020,7 @@
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1104.1</t>
+          <t>ICC A117.1-2017 §1004.1</t>
         </is>
       </c>
       <c r="G176" s="2" t="inlineStr">
@@ -7980,7 +8028,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H176" s="2" t="n"/>
+      <c r="H176" s="2" t="inlineStr">
+        <is>
+          <t>Section corrected Oct 15, 2026: A117.1-2017 recreation is Chapter 10.</t>
+        </is>
+      </c>
       <c r="I176" s="2" t="n"/>
       <c r="J176" s="2" t="n"/>
       <c r="K176" s="2" t="n"/>
@@ -11170,7 +11222,7 @@
       <c r="G258" s="2" t="n"/>
       <c r="H258" s="2" t="inlineStr">
         <is>
-          <t>Applies only to work permitted under the 2021 MBC. Applies to chargers installed under the 2021 Michigan Building Code. For older installations the count is shown as best practice.</t>
+          <t>Applies only to work permitted under the 2021 MBC. The 2021 IBC requires at least one per type of charger; Michigan's adopted text is still to be confirmed. Chargers serving Group R-2, R-3 and R-4 housing are exempt. Applies to chargers installed under the 2021 Michigan Building Code; for older installations the count is shown as best practice.</t>
         </is>
       </c>
     </row>
@@ -11200,11 +11252,19 @@
           <t>min 132</t>
         </is>
       </c>
-      <c r="F259" s="2" t="n"/>
-      <c r="G259" s="2" t="n"/>
+      <c r="F259" s="2" t="inlineStr">
+        <is>
+          <t>2021 MBC §1107.2</t>
+        </is>
+      </c>
+      <c r="G259" s="2" t="inlineStr">
+        <is>
+          <t>min 132</t>
+        </is>
+      </c>
       <c r="H259" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Best practice or safety item, not an accessibility requirement. </t>
+          <t xml:space="preserve">Applies only to work permitted under the 2021 MBC. </t>
         </is>
       </c>
     </row>
@@ -11234,11 +11294,19 @@
           <t>min 60</t>
         </is>
       </c>
-      <c r="F260" s="2" t="n"/>
-      <c r="G260" s="2" t="n"/>
+      <c r="F260" s="2" t="inlineStr">
+        <is>
+          <t>2021 MBC §1107.2</t>
+        </is>
+      </c>
+      <c r="G260" s="2" t="inlineStr">
+        <is>
+          <t>min 60</t>
+        </is>
+      </c>
       <c r="H260" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Best practice or safety item, not an accessibility requirement. </t>
+          <t xml:space="preserve">Applies only to work permitted under the 2021 MBC. </t>
         </is>
       </c>
     </row>
@@ -11640,11 +11708,15 @@
       <c r="E272" s="2" t="n"/>
       <c r="F272" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1102.1</t>
+          <t>ICC A117.1-2017 §1002.1</t>
         </is>
       </c>
       <c r="G272" s="2" t="n"/>
-      <c r="H272" s="2" t="n"/>
+      <c r="H272" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADA text checked online (Access Board text) on Oct 15, 2026. </t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" s="2" t="inlineStr">
@@ -11674,7 +11746,7 @@
       </c>
       <c r="F273" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1102.2</t>
+          <t>ICC A117.1-2017 §1002.2</t>
         </is>
       </c>
       <c r="G273" s="2" t="inlineStr">
@@ -11682,7 +11754,11 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H273" s="2" t="n"/>
+      <c r="H273" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADA text checked online (Access Board text) on Oct 15, 2026. </t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" s="2" t="inlineStr">
@@ -11712,7 +11788,7 @@
       </c>
       <c r="F274" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1102.3.1</t>
+          <t>ICC A117.1-2017 §1002.3.1</t>
         </is>
       </c>
       <c r="G274" s="2" t="inlineStr">
@@ -11750,7 +11826,7 @@
       </c>
       <c r="F275" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1102.3.2</t>
+          <t>ICC A117.1-2017 §1002.3.2</t>
         </is>
       </c>
       <c r="G275" s="2" t="inlineStr">
@@ -11788,7 +11864,7 @@
       </c>
       <c r="F276" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1102.4.5</t>
+          <t>ICC A117.1-2017 §1002.4.5</t>
         </is>
       </c>
       <c r="G276" s="2" t="inlineStr">
@@ -11796,7 +11872,11 @@
           <t>min 32</t>
         </is>
       </c>
-      <c r="H276" s="2" t="n"/>
+      <c r="H276" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADA text checked online (Access Board text) on Oct 15, 2026. </t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" s="2" t="inlineStr">
@@ -11826,7 +11906,7 @@
       </c>
       <c r="F277" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1102.4.2 and 1102.4.4</t>
+          <t>ICC A117.1-2017 §1002.4.2 and 1002.4.4</t>
         </is>
       </c>
       <c r="G277" s="2" t="inlineStr">
@@ -11864,7 +11944,7 @@
       </c>
       <c r="F278" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1102.4.7</t>
+          <t>ICC A117.1-2017 §1002.4.7</t>
         </is>
       </c>
       <c r="G278" s="2" t="inlineStr">
@@ -11874,7 +11954,7 @@
       </c>
       <c r="H278" s="2" t="inlineStr">
         <is>
-          <t>Required where the ride design allows a companion seat.</t>
+          <t>ADA text checked online (Access Board text) on Oct 15, 2026. Required where the ride interior is wider than 53 in, seats more than one rider, and the wheelchair space is not in the center (ADA 1002.4.7). Otherwise mark N/A.</t>
         </is>
       </c>
     </row>
@@ -11906,7 +11986,7 @@
       </c>
       <c r="F279" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1102.5.2</t>
+          <t>ICC A117.1-2017 §1002.5.2</t>
         </is>
       </c>
       <c r="G279" s="2" t="inlineStr">
@@ -11914,7 +11994,11 @@
           <t>min 14, max 24</t>
         </is>
       </c>
-      <c r="H279" s="2" t="n"/>
+      <c r="H279" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADA text checked online (Access Board text) on Oct 15, 2026. </t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" s="2" t="inlineStr">
@@ -11952,7 +12036,11 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H280" s="2" t="n"/>
+      <c r="H280" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADA text checked online (Access Board text) on Oct 15, 2026. </t>
+        </is>
+      </c>
     </row>
     <row r="281">
       <c r="A281" s="2" t="inlineStr">
@@ -11978,11 +12066,15 @@
       <c r="E281" s="2" t="n"/>
       <c r="F281" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1110</t>
+          <t>ICC A117.1-2017 §1010</t>
         </is>
       </c>
       <c r="G281" s="2" t="n"/>
-      <c r="H281" s="2" t="n"/>
+      <c r="H281" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADA text checked online (Access Board text) on Oct 15, 2026. </t>
+        </is>
+      </c>
     </row>
     <row r="282">
       <c r="A282" s="2" t="inlineStr">
@@ -12002,7 +12094,7 @@
       </c>
       <c r="D282" s="2" t="inlineStr">
         <is>
-          <t>ADA 2010 §206.2.13</t>
+          <t>ADA 2010 §206.2.2 and 243</t>
         </is>
       </c>
       <c r="E282" s="2" t="inlineStr">
@@ -12012,7 +12104,7 @@
       </c>
       <c r="F282" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1110</t>
+          <t>ICC A117.1-2017 §1010</t>
         </is>
       </c>
       <c r="G282" s="2" t="inlineStr">
@@ -12050,7 +12142,7 @@
       </c>
       <c r="F283" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1110.1</t>
+          <t>ICC A117.1-2017 §1010.1</t>
         </is>
       </c>
       <c r="G283" s="2" t="inlineStr">
@@ -12058,7 +12150,11 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H283" s="2" t="n"/>
+      <c r="H283" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADA text checked online (Access Board text) on Oct 15, 2026. </t>
+        </is>
+      </c>
     </row>
     <row r="284">
       <c r="A284" s="2" t="inlineStr">
@@ -12088,7 +12184,7 @@
       </c>
       <c r="F284" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1110.1</t>
+          <t>ICC A117.1-2017 §1010.1</t>
         </is>
       </c>
       <c r="G284" s="2" t="inlineStr">
@@ -12096,7 +12192,11 @@
           <t>max 2.08</t>
         </is>
       </c>
-      <c r="H284" s="2" t="n"/>
+      <c r="H284" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADA text checked online (Access Board text) on Oct 15, 2026. </t>
+        </is>
+      </c>
     </row>
     <row r="285">
       <c r="A285" s="2" t="inlineStr">
@@ -12136,7 +12236,7 @@
       </c>
       <c r="H285" s="2" t="inlineStr">
         <is>
-          <t>A readily removable bench may overlap the turning space (ADA 612.3 Exception).</t>
+          <t>ADA text checked online (Access Board text) on Oct 15, 2026. A readily removable bench may overlap the turning space (ADA 612.3 Exception).</t>
         </is>
       </c>
     </row>
@@ -12176,7 +12276,11 @@
           <t>min 42</t>
         </is>
       </c>
-      <c r="H286" s="2" t="n"/>
+      <c r="H286" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADA text checked online (Access Board text) on Oct 15, 2026. </t>
+        </is>
+      </c>
     </row>
     <row r="287">
       <c r="A287" s="2" t="inlineStr">
@@ -12214,7 +12318,11 @@
           <t>min 20, max 24</t>
         </is>
       </c>
-      <c r="H287" s="2" t="n"/>
+      <c r="H287" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADA text checked online (Access Board text) on Oct 15, 2026. </t>
+        </is>
+      </c>
     </row>
     <row r="288">
       <c r="A288" s="2" t="inlineStr">
@@ -12252,7 +12360,11 @@
           <t>min 17, max 19</t>
         </is>
       </c>
-      <c r="H288" s="2" t="n"/>
+      <c r="H288" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADA text checked online (Access Board text) on Oct 15, 2026. </t>
+        </is>
+      </c>
     </row>
     <row r="289">
       <c r="A289" s="2" t="inlineStr">
@@ -12290,7 +12402,11 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H289" s="2" t="n"/>
+      <c r="H289" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADA text checked online (Access Board text) on Oct 15, 2026. </t>
+        </is>
+      </c>
     </row>
     <row r="290">
       <c r="A290" s="2" t="inlineStr">
@@ -12328,7 +12444,11 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H290" s="2" t="n"/>
+      <c r="H290" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADA text checked online (Access Board text) on Oct 15, 2026. </t>
+        </is>
+      </c>
     </row>
     <row r="291">
       <c r="A291" s="2" t="inlineStr">
@@ -12366,7 +12486,11 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H291" s="2" t="n"/>
+      <c r="H291" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADA text checked online (Access Board text) on Oct 15, 2026. </t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Match ride, shooting and sauna rules to the ICC A117.1-2017 text
Amy shared the ICC A117.1-2017 pages for amusement rides, shooting facilities, saunas and benches. Michigan citations that match the text lose their dagger. Turning space at firing positions is A117.1 1010.2, load and unload areas are 1002.3, and the A117.1 34 in maximum firing counter height (1010.3) is added. Count and route rules point to the Michigan Building Code scoping sections instead.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AdurZhc4WrEcjZAJU4UBbC
</commit_message>
<xml_diff>
--- a/Rules review - Michigan citations to verify.xlsx
+++ b/Rules review - Michigan citations to verify.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L296"/>
+  <dimension ref="A1:L297"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -11708,13 +11708,13 @@
       <c r="E272" s="2" t="n"/>
       <c r="F272" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1002.1</t>
+          <t>2021 MBC §1110; ICC A117.1-2017 §1002.1</t>
         </is>
       </c>
       <c r="G272" s="2" t="n"/>
       <c r="H272" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADA text checked online (Access Board text) on Oct 15, 2026. </t>
+          <t xml:space="preserve">ADA text checked online (Access Board text), Oct 15, 2026. </t>
         </is>
       </c>
     </row>
@@ -11756,7 +11756,7 @@
       </c>
       <c r="H273" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADA text checked online (Access Board text) on Oct 15, 2026. </t>
+          <t xml:space="preserve">ADA text checked online (Access Board text), Oct 15, 2026. Michigan text matched against ICC A117.1-2017 pages from ICC Digital Codes, Oct 15, 2026. </t>
         </is>
       </c>
     </row>
@@ -11788,7 +11788,7 @@
       </c>
       <c r="F274" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1002.3.1</t>
+          <t>ICC A117.1-2017 §1002.3 and 304</t>
         </is>
       </c>
       <c r="G274" s="2" t="inlineStr">
@@ -11796,7 +11796,11 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H274" s="2" t="n"/>
+      <c r="H274" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Michigan text matched against ICC A117.1-2017 pages from ICC Digital Codes, Oct 15, 2026. </t>
+        </is>
+      </c>
     </row>
     <row r="275">
       <c r="A275" s="2" t="inlineStr">
@@ -11826,7 +11830,7 @@
       </c>
       <c r="F275" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1002.3.2</t>
+          <t>ICC A117.1-2017 §1002.3 and 304.2</t>
         </is>
       </c>
       <c r="G275" s="2" t="inlineStr">
@@ -11874,7 +11878,7 @@
       </c>
       <c r="H276" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADA text checked online (Access Board text) on Oct 15, 2026. </t>
+          <t xml:space="preserve">ADA text checked online (Access Board text), Oct 15, 2026. Michigan text matched against ICC A117.1-2017 pages from ICC Digital Codes, Oct 15, 2026. </t>
         </is>
       </c>
     </row>
@@ -11906,7 +11910,7 @@
       </c>
       <c r="F277" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1002.4.2 and 1002.4.4</t>
+          <t>ICC A117.1-2017 §1002.4.2 and 1002.4.4.1</t>
         </is>
       </c>
       <c r="G277" s="2" t="inlineStr">
@@ -11914,7 +11918,11 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H277" s="2" t="n"/>
+      <c r="H277" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Michigan text matched against ICC A117.1-2017 pages from ICC Digital Codes, Oct 15, 2026. </t>
+        </is>
+      </c>
     </row>
     <row r="278">
       <c r="A278" s="2" t="inlineStr">
@@ -11954,7 +11962,7 @@
       </c>
       <c r="H278" s="2" t="inlineStr">
         <is>
-          <t>ADA text checked online (Access Board text) on Oct 15, 2026. Required where the ride interior is wider than 53 in, seats more than one rider, and the wheelchair space is not in the center (ADA 1002.4.7). Otherwise mark N/A.</t>
+          <t>ADA text checked online (Access Board text), Oct 15, 2026. Michigan text matched against ICC A117.1-2017 pages from ICC Digital Codes, Oct 15, 2026. Required where the ride interior is wider than 53 in, seats more than one rider, and the wheelchair space is not in the center (ADA 1002.4.7). Otherwise mark N/A.</t>
         </is>
       </c>
     </row>
@@ -11996,7 +12004,7 @@
       </c>
       <c r="H279" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADA text checked online (Access Board text) on Oct 15, 2026. </t>
+          <t xml:space="preserve">ADA text checked online (Access Board text), Oct 15, 2026. Michigan text matched against ICC A117.1-2017 pages from ICC Digital Codes, Oct 15, 2026. </t>
         </is>
       </c>
     </row>
@@ -12038,7 +12046,7 @@
       </c>
       <c r="H280" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADA text checked online (Access Board text) on Oct 15, 2026. </t>
+          <t xml:space="preserve">ADA text checked online (Access Board text), Oct 15, 2026. </t>
         </is>
       </c>
     </row>
@@ -12066,13 +12074,13 @@
       <c r="E281" s="2" t="n"/>
       <c r="F281" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1010</t>
+          <t>2021 MBC §1110</t>
         </is>
       </c>
       <c r="G281" s="2" t="n"/>
       <c r="H281" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADA text checked online (Access Board text) on Oct 15, 2026. </t>
+          <t xml:space="preserve">ADA text checked online (Access Board text), Oct 15, 2026. </t>
         </is>
       </c>
     </row>
@@ -12104,7 +12112,7 @@
       </c>
       <c r="F282" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1010</t>
+          <t>2021 MBC §1104</t>
         </is>
       </c>
       <c r="G282" s="2" t="inlineStr">
@@ -12142,7 +12150,7 @@
       </c>
       <c r="F283" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1010.1</t>
+          <t>ICC A117.1-2017 §1010.2 and 304.3.1</t>
         </is>
       </c>
       <c r="G283" s="2" t="inlineStr">
@@ -12152,7 +12160,7 @@
       </c>
       <c r="H283" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADA text checked online (Access Board text) on Oct 15, 2026. </t>
+          <t xml:space="preserve">ADA text checked online (Access Board text), Oct 15, 2026. Michigan text matched against ICC A117.1-2017 pages from ICC Digital Codes, Oct 15, 2026. </t>
         </is>
       </c>
     </row>
@@ -12184,7 +12192,7 @@
       </c>
       <c r="F284" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §1010.1</t>
+          <t>ICC A117.1-2017 §1010.2</t>
         </is>
       </c>
       <c r="G284" s="2" t="inlineStr">
@@ -12194,49 +12202,41 @@
       </c>
       <c r="H284" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADA text checked online (Access Board text) on Oct 15, 2026. </t>
+          <t xml:space="preserve">ADA text checked online (Access Board text), Oct 15, 2026. Michigan text matched against ICC A117.1-2017 pages from ICC Digital Codes, Oct 15, 2026. </t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="2" t="inlineStr">
         <is>
-          <t>Sauna or steam room</t>
+          <t>Shooting range (firing positions)</t>
         </is>
       </c>
       <c r="B285" s="2" t="inlineStr">
         <is>
-          <t>Turning space</t>
+          <t>Counter or wall height where firing over it (34 in max)</t>
         </is>
       </c>
       <c r="C285" s="2" t="inlineStr">
         <is>
-          <t>bool</t>
-        </is>
-      </c>
-      <c r="D285" s="2" t="inlineStr">
-        <is>
-          <t>ADA 2010 §612.3</t>
-        </is>
-      </c>
-      <c r="E285" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D285" s="2" t="n"/>
+      <c r="E285" s="2" t="n"/>
       <c r="F285" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §612.3</t>
+          <t>ICC A117.1-2017 §1010.3</t>
         </is>
       </c>
       <c r="G285" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>max 34</t>
         </is>
       </c>
       <c r="H285" s="2" t="inlineStr">
         <is>
-          <t>ADA text checked online (Access Board text) on Oct 15, 2026. A readily removable bench may overlap the turning space (ADA 612.3 Exception).</t>
+          <t>Michigan text matched against ICC A117.1-2017 pages from ICC Digital Codes, Oct 15, 2026. Michigan (ICC A117.1) rule; the 2010 ADA Standards have no firing-counter height. Where other positions of the same type have counters, the accessible one needs an equivalent counter.</t>
         </is>
       </c>
     </row>
@@ -12248,37 +12248,37 @@
       </c>
       <c r="B286" s="2" t="inlineStr">
         <is>
-          <t>Bench length (42 in min)</t>
+          <t>Turning space</t>
         </is>
       </c>
       <c r="C286" s="2" t="inlineStr">
         <is>
-          <t>in</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="D286" s="2" t="inlineStr">
         <is>
-          <t>ADA 2010 §612.2 and 903.3</t>
+          <t>ADA 2010 §612.3</t>
         </is>
       </c>
       <c r="E286" s="2" t="inlineStr">
         <is>
-          <t>min 42</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="F286" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §612.2 and 903.3</t>
+          <t>ICC A117.1-2017 §612.3</t>
         </is>
       </c>
       <c r="G286" s="2" t="inlineStr">
         <is>
-          <t>min 42</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H286" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADA text checked online (Access Board text) on Oct 15, 2026. </t>
+          <t>ADA text checked online (Access Board text), Oct 15, 2026. Michigan text matched against ICC A117.1-2017 pages from ICC Digital Codes, Oct 15, 2026. Under the ADA a readily removable bench may overlap the turning space (ADA 612.3 Exception). ICC A117.1 has no such exception, but lets door and bench clearances overlap the turning space.</t>
         </is>
       </c>
     </row>
@@ -12290,7 +12290,7 @@
       </c>
       <c r="B287" s="2" t="inlineStr">
         <is>
-          <t>Bench depth (20 to 24 in)</t>
+          <t>Bench length (42 in min)</t>
         </is>
       </c>
       <c r="C287" s="2" t="inlineStr">
@@ -12305,7 +12305,7 @@
       </c>
       <c r="E287" s="2" t="inlineStr">
         <is>
-          <t>min 20, max 24</t>
+          <t>min 42</t>
         </is>
       </c>
       <c r="F287" s="2" t="inlineStr">
@@ -12315,12 +12315,12 @@
       </c>
       <c r="G287" s="2" t="inlineStr">
         <is>
-          <t>min 20, max 24</t>
+          <t>min 42</t>
         </is>
       </c>
       <c r="H287" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADA text checked online (Access Board text) on Oct 15, 2026. </t>
+          <t xml:space="preserve">ADA text checked online (Access Board text), Oct 15, 2026. Michigan text matched against ICC A117.1-2017 pages from ICC Digital Codes, Oct 15, 2026. </t>
         </is>
       </c>
     </row>
@@ -12332,7 +12332,7 @@
       </c>
       <c r="B288" s="2" t="inlineStr">
         <is>
-          <t>Bench height (17 to 19 in)</t>
+          <t>Bench depth (20 to 24 in)</t>
         </is>
       </c>
       <c r="C288" s="2" t="inlineStr">
@@ -12342,27 +12342,27 @@
       </c>
       <c r="D288" s="2" t="inlineStr">
         <is>
-          <t>ADA 2010 §612.2 and 903.5</t>
+          <t>ADA 2010 §612.2 and 903.3</t>
         </is>
       </c>
       <c r="E288" s="2" t="inlineStr">
         <is>
-          <t>min 17, max 19</t>
+          <t>min 20, max 24</t>
         </is>
       </c>
       <c r="F288" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §612.2 and 903.5</t>
+          <t>ICC A117.1-2017 §612.2 and 903.3</t>
         </is>
       </c>
       <c r="G288" s="2" t="inlineStr">
         <is>
-          <t>min 17, max 19</t>
+          <t>min 20, max 24</t>
         </is>
       </c>
       <c r="H288" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADA text checked online (Access Board text) on Oct 15, 2026. </t>
+          <t xml:space="preserve">ADA text checked online (Access Board text), Oct 15, 2026. Michigan text matched against ICC A117.1-2017 pages from ICC Digital Codes, Oct 15, 2026. </t>
         </is>
       </c>
     </row>
@@ -12374,37 +12374,37 @@
       </c>
       <c r="B289" s="2" t="inlineStr">
         <is>
-          <t>Back support</t>
+          <t>Bench height (17 to 19 in)</t>
         </is>
       </c>
       <c r="C289" s="2" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>in</t>
         </is>
       </c>
       <c r="D289" s="2" t="inlineStr">
         <is>
-          <t>ADA 2010 §612.2 and 903.4</t>
+          <t>ADA 2010 §612.2 and 903.5</t>
         </is>
       </c>
       <c r="E289" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>min 17, max 19</t>
         </is>
       </c>
       <c r="F289" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §612.2 and 903.4</t>
+          <t>ICC A117.1-2017 §612.2 and 903.5</t>
         </is>
       </c>
       <c r="G289" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>min 17, max 19</t>
         </is>
       </c>
       <c r="H289" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADA text checked online (Access Board text) on Oct 15, 2026. </t>
+          <t xml:space="preserve">ADA text checked online (Access Board text), Oct 15, 2026. Michigan text matched against ICC A117.1-2017 pages from ICC Digital Codes, Oct 15, 2026. </t>
         </is>
       </c>
     </row>
@@ -12416,7 +12416,7 @@
       </c>
       <c r="B290" s="2" t="inlineStr">
         <is>
-          <t>Clear floor space at the bench</t>
+          <t>Back support</t>
         </is>
       </c>
       <c r="C290" s="2" t="inlineStr">
@@ -12426,7 +12426,7 @@
       </c>
       <c r="D290" s="2" t="inlineStr">
         <is>
-          <t>ADA 2010 §612.2 and 903.2</t>
+          <t>ADA 2010 §612.2 and 903.4</t>
         </is>
       </c>
       <c r="E290" s="2" t="inlineStr">
@@ -12436,7 +12436,7 @@
       </c>
       <c r="F290" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §612.2 and 903.2</t>
+          <t>ICC A117.1-2017 §612.2 and 903.4</t>
         </is>
       </c>
       <c r="G290" s="2" t="inlineStr">
@@ -12446,7 +12446,7 @@
       </c>
       <c r="H290" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADA text checked online (Access Board text) on Oct 15, 2026. </t>
+          <t xml:space="preserve">ADA text checked online (Access Board text), Oct 15, 2026. Michigan text matched against ICC A117.1-2017 pages from ICC Digital Codes, Oct 15, 2026. </t>
         </is>
       </c>
     </row>
@@ -12458,7 +12458,7 @@
       </c>
       <c r="B291" s="2" t="inlineStr">
         <is>
-          <t>Door does not swing into the bench clear floor space</t>
+          <t>Clear floor space at the bench</t>
         </is>
       </c>
       <c r="C291" s="2" t="inlineStr">
@@ -12468,7 +12468,7 @@
       </c>
       <c r="D291" s="2" t="inlineStr">
         <is>
-          <t>ADA 2010 §612.2</t>
+          <t>ADA 2010 §612.2 and 903.2</t>
         </is>
       </c>
       <c r="E291" s="2" t="inlineStr">
@@ -12478,7 +12478,7 @@
       </c>
       <c r="F291" s="2" t="inlineStr">
         <is>
-          <t>ICC A117.1-2017 §612.2</t>
+          <t>ICC A117.1-2017 §612.2 and 903.2</t>
         </is>
       </c>
       <c r="G291" s="2" t="inlineStr">
@@ -12488,19 +12488,19 @@
       </c>
       <c r="H291" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADA text checked online (Access Board text) on Oct 15, 2026. </t>
+          <t xml:space="preserve">ADA text checked online (Access Board text), Oct 15, 2026. Michigan text matched against ICC A117.1-2017 pages from ICC Digital Codes, Oct 15, 2026. </t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="2" t="inlineStr">
         <is>
-          <t>Playground safety check (not accessibility)</t>
+          <t>Sauna or steam room</t>
         </is>
       </c>
       <c r="B292" s="2" t="inlineStr">
         <is>
-          <t>Protective surfacing</t>
+          <t>Door does not swing into the bench clear floor space</t>
         </is>
       </c>
       <c r="C292" s="2" t="inlineStr">
@@ -12510,7 +12510,7 @@
       </c>
       <c r="D292" s="2" t="inlineStr">
         <is>
-          <t>CPSC Public Playground Safety Handbook, adopted by Michigan's Playground Equipment Safety Act (1997 PA 16)</t>
+          <t>ADA 2010 §612.2</t>
         </is>
       </c>
       <c r="E292" s="2" t="inlineStr">
@@ -12518,11 +12518,19 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="F292" s="2" t="n"/>
-      <c r="G292" s="2" t="n"/>
+      <c r="F292" s="2" t="inlineStr">
+        <is>
+          <t>ICC A117.1-2017 §612.2</t>
+        </is>
+      </c>
+      <c r="G292" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="H292" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Best practice or safety item, not an accessibility requirement. </t>
+          <t>ADA text checked online (Access Board text), Oct 15, 2026. Michigan text matched against ICC A117.1-2017 pages from ICC Digital Codes, Oct 15, 2026. Michigan (ICC A117.1 612.2 Exception): in a single-user room the door may swing over the bench space if a 30 x 48 in clear floor space is left beyond the door swing.</t>
         </is>
       </c>
     </row>
@@ -12534,7 +12542,7 @@
       </c>
       <c r="B293" s="2" t="inlineStr">
         <is>
-          <t>Use zones clear (6 ft min)</t>
+          <t>Protective surfacing</t>
         </is>
       </c>
       <c r="C293" s="2" t="inlineStr">
@@ -12568,7 +12576,7 @@
       </c>
       <c r="B294" s="2" t="inlineStr">
         <is>
-          <t>No head entrapment openings</t>
+          <t>Use zones clear (6 ft min)</t>
         </is>
       </c>
       <c r="C294" s="2" t="inlineStr">
@@ -12602,7 +12610,7 @@
       </c>
       <c r="B295" s="2" t="inlineStr">
         <is>
-          <t>Equipment in good repair</t>
+          <t>No head entrapment openings</t>
         </is>
       </c>
       <c r="C295" s="2" t="inlineStr">
@@ -12636,7 +12644,7 @@
       </c>
       <c r="B296" s="2" t="inlineStr">
         <is>
-          <t>Inspection record</t>
+          <t>Equipment in good repair</t>
         </is>
       </c>
       <c r="C296" s="2" t="inlineStr">
@@ -12657,6 +12665,40 @@
       <c r="F296" s="2" t="n"/>
       <c r="G296" s="2" t="n"/>
       <c r="H296" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Best practice or safety item, not an accessibility requirement. </t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="2" t="inlineStr">
+        <is>
+          <t>Playground safety check (not accessibility)</t>
+        </is>
+      </c>
+      <c r="B297" s="2" t="inlineStr">
+        <is>
+          <t>Inspection record</t>
+        </is>
+      </c>
+      <c r="C297" s="2" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="D297" s="2" t="inlineStr">
+        <is>
+          <t>CPSC Public Playground Safety Handbook, adopted by Michigan's Playground Equipment Safety Act (1997 PA 16)</t>
+        </is>
+      </c>
+      <c r="E297" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F297" s="2" t="n"/>
+      <c r="G297" s="2" t="n"/>
+      <c r="H297" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Best practice or safety item, not an accessibility requirement. </t>
         </is>

</xml_diff>